<commit_message>
looking through the data that already exists to see what the dealio is.
</commit_message>
<xml_diff>
--- a/CleanData/DataDictionary.xlsx
+++ b/CleanData/DataDictionary.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ainsl/Desktop/R01_Aim1H1/CleanData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF33C886-2E25-1843-88BF-6289B4D657C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4626FE-89E2-3C42-9969-697E28716E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3720" yWindow="1660" windowWidth="21560" windowHeight="15600" activeTab="1" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
+    <workbookView xWindow="16120" yWindow="760" windowWidth="15800" windowHeight="16640" activeTab="1" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
   </bookViews>
   <sheets>
     <sheet name="CleanedData" sheetId="1" r:id="rId1"/>
     <sheet name="ALCUSE Data" sheetId="2" r:id="rId2"/>
     <sheet name="R6_2 Data" sheetId="3" r:id="rId3"/>
+    <sheet name="SelfReported_DrinkingDriving" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="339">
   <si>
     <t>Variable</t>
   </si>
@@ -476,9 +477,6 @@
     <t>Primary CV Sample Type</t>
   </si>
   <si>
-    <t>/R01_Aim1H1/RawData/ALCUSE.dat</t>
-  </si>
-  <si>
     <t>S0922200</t>
   </si>
   <si>
@@ -837,13 +835,391 @@
   </si>
   <si>
     <t>Data located in /R01_Aim1H1/RawData/ALCUSE.dat</t>
+  </si>
+  <si>
+    <t>Data located in /R01_Aim1H1/RawData/R6_2.dat</t>
+  </si>
+  <si>
+    <t>KEY_SEX_1997</t>
+  </si>
+  <si>
+    <t>KEY!SEX (SYMBOL) 1997</t>
+  </si>
+  <si>
+    <t>KEY_BDATE_M_1997</t>
+  </si>
+  <si>
+    <t>KEY!BDATE M/Y (SYMBOL) 1997</t>
+  </si>
+  <si>
+    <t>KEY_BDATE_Y_1997</t>
+  </si>
+  <si>
+    <t>KEY_ETHNICITY_1997</t>
+  </si>
+  <si>
+    <t>KEY!ETHNICITY (SYMBOL) 1997</t>
+  </si>
+  <si>
+    <t>KEY_RACE_1997</t>
+  </si>
+  <si>
+    <t>KEY!RACE (SYMBOL) 1997</t>
+  </si>
+  <si>
+    <t>CV_CITIZENSHIP_1997</t>
+  </si>
+  <si>
+    <t>CV_CITIZENSHIP 1997</t>
+  </si>
+  <si>
+    <t>CV_INCOME_GROSS_YR_1997</t>
+  </si>
+  <si>
+    <t>Continuous</t>
+  </si>
+  <si>
+    <t>CV_INCOME_GROSS_YR 1997</t>
+  </si>
+  <si>
+    <t>CV_HH_NET_WORTH_P_1997</t>
+  </si>
+  <si>
+    <t>CV_HH_NET_WORTH_P 1997</t>
+  </si>
+  <si>
+    <t>CV_HH_POV_RATIO_1997</t>
+  </si>
+  <si>
+    <t>CV_HH_POV_RATIO 1997</t>
+  </si>
+  <si>
+    <t>CV_SAMPLE_TYPE_1997</t>
+  </si>
+  <si>
+    <t>CV_SAMPLE_TYPE 1997</t>
+  </si>
+  <si>
+    <t>CV_HGC_BIO_DAD_1997</t>
+  </si>
+  <si>
+    <t>CV_HGC_BIO_DAD 1997</t>
+  </si>
+  <si>
+    <t>CV_HGC_BIO_MOM_1997</t>
+  </si>
+  <si>
+    <t>CV_HGC_BIO_MOM 1997</t>
+  </si>
+  <si>
+    <t>CV_HGC_RES_DAD_1997</t>
+  </si>
+  <si>
+    <t>CV_HGC_RES_DAD 1997</t>
+  </si>
+  <si>
+    <t>CV_HGC_RES_MOM_1997</t>
+  </si>
+  <si>
+    <t>CV_HGC_RES_MOM 1997</t>
+  </si>
+  <si>
+    <t>KEY_RACE_ETHNICITY_1997</t>
+  </si>
+  <si>
+    <t>KEY!RACE_ETHNICITY (SYMBOL) 1997</t>
+  </si>
+  <si>
+    <t>FP_YMMONIT_1997</t>
+  </si>
+  <si>
+    <t>MONITOR BY RES MOM, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_YFMONIT_1997</t>
+  </si>
+  <si>
+    <t>MONITOR BY RES DAD, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_YNRMMONIT_1997</t>
+  </si>
+  <si>
+    <t>MONITOR BY NON-RES MOM, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_YNRFMONIT_1997</t>
+  </si>
+  <si>
+    <t>MONITOR BY NON-RES DAD, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_YHLIMITS_1997</t>
+  </si>
+  <si>
+    <t>AUTONOMY AND CONTROL, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_PHLIMITS_1997</t>
+  </si>
+  <si>
+    <t>AUTONOMY AND CONTROL, PAR RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_YHBROKED_1997</t>
+  </si>
+  <si>
+    <t>LIMIT-BREAKING, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_PHBROKED_1997</t>
+  </si>
+  <si>
+    <t>LIMIT-BREAKING, PAR RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_YMPSTYL_1997</t>
+  </si>
+  <si>
+    <t>RES MOM'S PARENT STYLE, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_YFPSTYL_1997</t>
+  </si>
+  <si>
+    <t>RES DAD'S PARENT STYLE, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_YNRMPSTYL_1997</t>
+  </si>
+  <si>
+    <t>NON-RES MOM'S PARENT STYLE, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_YNRFPSTYL_1997</t>
+  </si>
+  <si>
+    <t>NON-RES DAD'S PARENT STYLE, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_PPRELIG_1997</t>
+  </si>
+  <si>
+    <t>PARENT'S RELIGIOSITY, PARENT REPORT 1997</t>
+  </si>
+  <si>
+    <t>FP_ADHRISKI_1997</t>
+  </si>
+  <si>
+    <t>FAMILY/HOME RISK INDEX 1997</t>
+  </si>
+  <si>
+    <t>FP_ADPENVRI_1997</t>
+  </si>
+  <si>
+    <t>PHYSICAL ENVIRONMENT RISK INDEX 1997</t>
+  </si>
+  <si>
+    <t>FP_ADENRCHI_1997</t>
+  </si>
+  <si>
+    <t>ENRICHING ENVIRONMENT RISK INDEX 1997</t>
+  </si>
+  <si>
+    <t>FP_YYFBEHS_1997</t>
+  </si>
+  <si>
+    <t>GIRLS BEHAVE/EMOT SCALE, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_YYMBEHS_1997</t>
+  </si>
+  <si>
+    <t>BOYS BEHAVE/EMOT SCALE, YTH RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_PYFBEHS_1997</t>
+  </si>
+  <si>
+    <t>GIRLS BEHAVE/EMOT SCALE, PAR RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_PYMBEHS_1997</t>
+  </si>
+  <si>
+    <t>BOYS BEHAVE/EMOT SCALE, PAR RPT 1997</t>
+  </si>
+  <si>
+    <t>FP_YYCRIMI_1997</t>
+  </si>
+  <si>
+    <t>DELINQUENCY SCORE INDEX 1997</t>
+  </si>
+  <si>
+    <t>FP_YYSUBSI_1997</t>
+  </si>
+  <si>
+    <t>SUBSTANCE USE INDEX 1997</t>
+  </si>
+  <si>
+    <t>YSCH-2857_2002</t>
+  </si>
+  <si>
+    <t>WHAT IS CURR HGA? 2002</t>
+  </si>
+  <si>
+    <t>YSCH-3112_2002</t>
+  </si>
+  <si>
+    <t>WHAT IS CURR HGC? 2002</t>
+  </si>
+  <si>
+    <t>YSAQ-360C_2002</t>
+  </si>
+  <si>
+    <t>R SMOKED SDLI? 2002</t>
+  </si>
+  <si>
+    <t>YSAQ-361_2002</t>
+  </si>
+  <si>
+    <t># DAYS SMOKED LAST 30 DAYS 2002</t>
+  </si>
+  <si>
+    <t>YSAQ-362_2002</t>
+  </si>
+  <si>
+    <t># CIGS SMOKED/DAY LAST 30 DAYS 2002</t>
+  </si>
+  <si>
+    <t>YSAQ-372B_2002</t>
+  </si>
+  <si>
+    <t>R EVER USE OTH DRUGS? 2002</t>
+  </si>
+  <si>
+    <t>YSAQ-372C_2002</t>
+  </si>
+  <si>
+    <t>AGE 1ST TIME USE OTH DRUGS? 2002</t>
+  </si>
+  <si>
+    <t>YSAQ-372CC_2002</t>
+  </si>
+  <si>
+    <t>R USE COC/DRUGS SDLI? 2002</t>
+  </si>
+  <si>
+    <t>YSAQ-372D_2002</t>
+  </si>
+  <si>
+    <t># TIMES USE COC/DRUGS SDLI? 2002</t>
+  </si>
+  <si>
+    <t>YSAQ-372E_2002</t>
+  </si>
+  <si>
+    <t># TIMES COC/DRUGS DUR SCH/WRK 2002</t>
+  </si>
+  <si>
+    <t>YINC-1400_2002</t>
+  </si>
+  <si>
+    <t>R RCV INC FROM JOB PAST YR? 2002</t>
+  </si>
+  <si>
+    <t>YINC-1500_2002</t>
+  </si>
+  <si>
+    <t>INC WAGE, TIPS REG/ODD JOBS? 2002</t>
+  </si>
+  <si>
+    <t>YINC-1700_2002</t>
+  </si>
+  <si>
+    <t>TTL INC WAGES, SALARY PAST YR 2002</t>
+  </si>
+  <si>
+    <t>YINC-1800_2002</t>
+  </si>
+  <si>
+    <t>EST INC WAGES, TIPS PAST YR 2002</t>
+  </si>
+  <si>
+    <t>YINC-2600_2002</t>
+  </si>
+  <si>
+    <t>SP TTL INC WAGES, SALARY PAST YR 2002</t>
+  </si>
+  <si>
+    <t>YINC-2700_2002</t>
+  </si>
+  <si>
+    <t>EST SP INC WAGE, SAL PAST YR 2002</t>
+  </si>
+  <si>
+    <t>YHEA-650_2002</t>
+  </si>
+  <si>
+    <t>HRS/NIGHT R SLEEPS 2002</t>
+  </si>
+  <si>
+    <t>Net worth of the respondent's household according to parent</t>
+  </si>
+  <si>
+    <t>Calculated total household income in previous calendar year</t>
+  </si>
+  <si>
+    <t>Describe the parenting styles--uninvolved, permissive, authoritarian, and authoritative--of youth's parents/parent-figures.</t>
+  </si>
+  <si>
+    <t>Describe the awareness of the youth's activities for up to four parents/parent-figures in rounds 1-4. Scores range from 0 to 16</t>
+  </si>
+  <si>
+    <t>'R0536401',</t>
+  </si>
+  <si>
+    <t>'R0536402',</t>
+  </si>
+  <si>
+    <t>'R1235800',</t>
+  </si>
+  <si>
+    <t>'R1482600',</t>
+  </si>
+  <si>
+    <t>'T1050200',</t>
+  </si>
+  <si>
+    <t>'T3145400',</t>
+  </si>
+  <si>
+    <t>'T4565700',</t>
+  </si>
+  <si>
+    <t>'T6209900',</t>
+  </si>
+  <si>
+    <t>'T7707300',</t>
+  </si>
+  <si>
+    <t>'U1100000',</t>
+  </si>
+  <si>
+    <t>U2963200'</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>S1542400</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -897,8 +1273,23 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -917,8 +1308,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1014,11 +1411,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1064,6 +1476,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1072,8 +1494,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFDEEDFE"/>
       <color rgb="FFFFF7F8"/>
-      <color rgb="FFDEEDFE"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1404,7 +1826,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A5CC42-7E80-3145-82C3-AE1AB4759DCA}">
-  <dimension ref="A1:I147"/>
+  <dimension ref="A1:I142"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" customWidth="1"/>
@@ -1690,6 +2112,9 @@
       <c r="D18" s="11" t="s">
         <v>26</v>
       </c>
+      <c r="E18" t="s">
+        <v>338</v>
+      </c>
     </row>
     <row r="19" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="18" t="s">
@@ -1848,105 +2273,67 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="18"/>
-      <c r="B28" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="C28" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="D28" s="18" t="s">
-        <v>102</v>
-      </c>
+      <c r="B28" s="19"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
       <c r="E28" s="18" t="s">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G28" s="18"/>
       <c r="H28" s="18"/>
       <c r="I28" s="18"/>
     </row>
-    <row r="29" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="18"/>
-      <c r="B29" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="C29" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="D29" s="18" t="s">
-        <v>103</v>
-      </c>
+      <c r="B29" s="19"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
       <c r="E29" s="18" t="s">
-        <v>94</v>
-      </c>
-      <c r="F29" s="18" t="s">
-        <v>93</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="F29" s="18"/>
       <c r="G29" s="18"/>
       <c r="H29" s="18"/>
       <c r="I29" s="18"/>
     </row>
-    <row r="30" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="18"/>
-      <c r="B30" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="C30" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="D30" s="18" t="s">
-        <v>105</v>
-      </c>
+      <c r="B30" s="19"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
       <c r="E30" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="F30" s="18" t="s">
-        <v>93</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="F30" s="18"/>
       <c r="G30" s="18"/>
       <c r="H30" s="18"/>
       <c r="I30" s="18"/>
     </row>
-    <row r="31" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="18"/>
-      <c r="B31" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="C31" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="D31" s="18" t="s">
-        <v>104</v>
-      </c>
+      <c r="B31" s="19"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
       <c r="E31" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="F31" s="18" t="s">
-        <v>93</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="F31" s="18"/>
       <c r="G31" s="18"/>
       <c r="H31" s="18"/>
       <c r="I31" s="18"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="18"/>
-      <c r="B32" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="C32" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="D32" s="18" t="s">
-        <v>105</v>
-      </c>
+      <c r="B32" s="19"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
       <c r="E32" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="F32" s="18" t="s">
-        <v>93</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="F32" s="18"/>
       <c r="G32" s="18"/>
       <c r="H32" s="18"/>
       <c r="I32" s="18"/>
@@ -1957,11 +2344,9 @@
       <c r="C33" s="18"/>
       <c r="D33" s="18"/>
       <c r="E33" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="F33" s="18" t="s">
-        <v>106</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="F33" s="18"/>
       <c r="G33" s="18"/>
       <c r="H33" s="18"/>
       <c r="I33" s="18"/>
@@ -1972,7 +2357,7 @@
       <c r="C34" s="18"/>
       <c r="D34" s="18"/>
       <c r="E34" s="18" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F34" s="18"/>
       <c r="G34" s="18"/>
@@ -1985,7 +2370,7 @@
       <c r="C35" s="18"/>
       <c r="D35" s="18"/>
       <c r="E35" s="18" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F35" s="18"/>
       <c r="G35" s="18"/>
@@ -1998,7 +2383,7 @@
       <c r="C36" s="18"/>
       <c r="D36" s="18"/>
       <c r="E36" s="18" t="s">
-        <v>62</v>
+        <v>111</v>
       </c>
       <c r="F36" s="18"/>
       <c r="G36" s="18"/>
@@ -2011,7 +2396,7 @@
       <c r="C37" s="18"/>
       <c r="D37" s="18"/>
       <c r="E37" s="18" t="s">
-        <v>61</v>
+        <v>91</v>
       </c>
       <c r="F37" s="18"/>
       <c r="G37" s="18"/>
@@ -2024,7 +2409,7 @@
       <c r="C38" s="18"/>
       <c r="D38" s="18"/>
       <c r="E38" s="18" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F38" s="18"/>
       <c r="G38" s="18"/>
@@ -2037,7 +2422,7 @@
       <c r="C39" s="18"/>
       <c r="D39" s="18"/>
       <c r="E39" s="18" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="F39" s="18"/>
       <c r="G39" s="18"/>
@@ -2050,7 +2435,7 @@
       <c r="C40" s="18"/>
       <c r="D40" s="18"/>
       <c r="E40" s="18" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="F40" s="18"/>
       <c r="G40" s="18"/>
@@ -2063,7 +2448,7 @@
       <c r="C41" s="18"/>
       <c r="D41" s="18"/>
       <c r="E41" s="18" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F41" s="18"/>
       <c r="G41" s="18"/>
@@ -2076,7 +2461,7 @@
       <c r="C42" s="18"/>
       <c r="D42" s="18"/>
       <c r="E42" s="18" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="F42" s="18"/>
       <c r="G42" s="18"/>
@@ -2089,7 +2474,7 @@
       <c r="C43" s="18"/>
       <c r="D43" s="18"/>
       <c r="E43" s="18" t="s">
-        <v>113</v>
+        <v>59</v>
       </c>
       <c r="F43" s="18"/>
       <c r="G43" s="18"/>
@@ -2102,7 +2487,7 @@
       <c r="C44" s="18"/>
       <c r="D44" s="18"/>
       <c r="E44" s="18" t="s">
-        <v>114</v>
+        <v>58</v>
       </c>
       <c r="F44" s="18"/>
       <c r="G44" s="18"/>
@@ -2115,7 +2500,7 @@
       <c r="C45" s="18"/>
       <c r="D45" s="18"/>
       <c r="E45" s="18" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F45" s="18"/>
       <c r="G45" s="18"/>
@@ -2128,7 +2513,7 @@
       <c r="C46" s="18"/>
       <c r="D46" s="18"/>
       <c r="E46" s="18" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F46" s="18"/>
       <c r="G46" s="18"/>
@@ -2141,7 +2526,7 @@
       <c r="C47" s="18"/>
       <c r="D47" s="18"/>
       <c r="E47" s="18" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F47" s="18"/>
       <c r="G47" s="18"/>
@@ -2154,7 +2539,7 @@
       <c r="C48" s="18"/>
       <c r="D48" s="18"/>
       <c r="E48" s="18" t="s">
-        <v>59</v>
+        <v>120</v>
       </c>
       <c r="F48" s="18"/>
       <c r="G48" s="18"/>
@@ -2162,683 +2547,633 @@
       <c r="I48" s="18"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A49" s="18"/>
-      <c r="B49" s="19"/>
-      <c r="C49" s="18"/>
-      <c r="D49" s="18"/>
-      <c r="E49" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="F49" s="18"/>
+      <c r="A49" s="12"/>
+      <c r="E49" s="20" t="s">
+        <v>121</v>
+      </c>
       <c r="G49" s="18"/>
       <c r="H49" s="18"/>
       <c r="I49" s="18"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A50" s="18"/>
-      <c r="B50" s="19"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="18"/>
-      <c r="E50" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="F50" s="18"/>
+      <c r="A50" s="12"/>
+      <c r="E50" t="s">
+        <v>122</v>
+      </c>
       <c r="G50" s="18"/>
       <c r="H50" s="18"/>
       <c r="I50" s="18"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A51" s="18"/>
-      <c r="B51" s="19"/>
-      <c r="C51" s="18"/>
-      <c r="D51" s="18"/>
-      <c r="E51" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="F51" s="18"/>
+      <c r="A51" s="12"/>
+      <c r="E51" t="s">
+        <v>123</v>
+      </c>
       <c r="G51" s="18"/>
       <c r="H51" s="18"/>
       <c r="I51" s="18"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A52" s="18"/>
-      <c r="B52" s="19"/>
-      <c r="C52" s="18"/>
-      <c r="D52" s="18"/>
-      <c r="E52" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="F52" s="18"/>
+      <c r="A52" s="12"/>
+      <c r="E52" t="s">
+        <v>124</v>
+      </c>
       <c r="G52" s="18"/>
       <c r="H52" s="18"/>
       <c r="I52" s="18"/>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A53" s="18"/>
-      <c r="B53" s="19"/>
-      <c r="C53" s="18"/>
-      <c r="D53" s="18"/>
-      <c r="E53" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="F53" s="18"/>
+      <c r="A53" s="12"/>
+      <c r="E53" t="s">
+        <v>125</v>
+      </c>
       <c r="G53" s="18"/>
       <c r="H53" s="18"/>
       <c r="I53" s="18"/>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" s="12"/>
-      <c r="E54" s="20" t="s">
-        <v>122</v>
+      <c r="E54" t="s">
+        <v>126</v>
       </c>
       <c r="H54" s="13"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" s="12"/>
       <c r="E55" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="H55" s="13"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" s="12"/>
       <c r="E56" t="s">
-        <v>124</v>
+        <v>85</v>
       </c>
       <c r="H56" s="13"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" s="12"/>
       <c r="E57" t="s">
-        <v>125</v>
+        <v>84</v>
       </c>
       <c r="H57" s="13"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="12"/>
       <c r="E58" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H58" s="13"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" s="12"/>
       <c r="E59" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H59" s="13"/>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" s="12"/>
       <c r="E60" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H60" s="13"/>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" s="12"/>
       <c r="E61" t="s">
-        <v>85</v>
+        <v>131</v>
       </c>
       <c r="H61" s="13"/>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" s="12"/>
       <c r="E62" t="s">
-        <v>84</v>
+        <v>132</v>
       </c>
       <c r="H62" s="13"/>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" s="12"/>
       <c r="E63" t="s">
-        <v>129</v>
+        <v>86</v>
       </c>
       <c r="H63" s="13"/>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" s="12"/>
       <c r="E64" t="s">
-        <v>130</v>
+        <v>87</v>
       </c>
       <c r="H64" s="13"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="12"/>
       <c r="E65" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H65" s="13"/>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" s="12"/>
       <c r="E66" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H66" s="13"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="12"/>
       <c r="E67" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H67" s="13"/>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="12"/>
       <c r="E68" t="s">
-        <v>86</v>
+        <v>136</v>
       </c>
       <c r="H68" s="13"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="12"/>
       <c r="E69" t="s">
-        <v>87</v>
+        <v>137</v>
       </c>
       <c r="H69" s="13"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" s="12"/>
       <c r="E70" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="H70" s="13"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" s="12"/>
       <c r="E71" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="H71" s="13"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" s="12"/>
       <c r="E72" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="H72" s="13"/>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" s="12"/>
       <c r="E73" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="H73" s="13"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" s="12"/>
       <c r="E74" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="H74" s="13"/>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" s="12"/>
       <c r="E75" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="H75" s="13"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="12"/>
       <c r="E76" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="H76" s="13"/>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" s="12"/>
       <c r="E77" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="H77" s="13"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" s="12"/>
       <c r="E78" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="H78" s="13"/>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" s="12"/>
       <c r="E79" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="H79" s="13"/>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" s="12"/>
       <c r="E80" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="H80" s="13"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" s="12"/>
       <c r="E81" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="H81" s="13"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A82" s="12"/>
       <c r="E82" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="H82" s="13"/>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" s="12"/>
       <c r="E83" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="H83" s="13"/>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84" s="12"/>
       <c r="E84" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="H84" s="13"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="12"/>
       <c r="E85" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="H85" s="13"/>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86" s="12"/>
       <c r="E86" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="H86" s="13"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="12"/>
       <c r="E87" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="H87" s="13"/>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" s="12"/>
       <c r="E88" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="H88" s="13"/>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" s="12"/>
       <c r="E89" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="H89" s="13"/>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" s="12"/>
       <c r="E90" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H90" s="13"/>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91" s="12"/>
       <c r="E91" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="H91" s="13"/>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" s="12"/>
       <c r="E92" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="H92" s="13"/>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A93" s="12"/>
       <c r="E93" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="H93" s="13"/>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" s="12"/>
       <c r="E94" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="H94" s="13"/>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A95" s="12"/>
       <c r="E95" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="H95" s="13"/>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A96" s="12"/>
       <c r="E96" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="H96" s="13"/>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A97" s="12"/>
       <c r="E97" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="H97" s="13"/>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98" s="12"/>
       <c r="E98" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="H98" s="13"/>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A99" s="12"/>
       <c r="E99" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="H99" s="13"/>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A100" s="12"/>
       <c r="E100" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="H100" s="13"/>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A101" s="12"/>
       <c r="E101" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="H101" s="13"/>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A102" s="12"/>
       <c r="E102" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="H102" s="13"/>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A103" s="12"/>
       <c r="E103" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="H103" s="13"/>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A104" s="12"/>
       <c r="E104" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="H104" s="13"/>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A105" s="12"/>
       <c r="E105" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="H105" s="13"/>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A106" s="12"/>
       <c r="E106" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="H106" s="13"/>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A107" s="12"/>
       <c r="E107" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="H107" s="13"/>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A108" s="12"/>
       <c r="E108" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="H108" s="13"/>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A109" s="12"/>
       <c r="E109" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="H109" s="13"/>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A110" s="12"/>
       <c r="E110" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="H110" s="13"/>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A111" s="12"/>
       <c r="E111" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="H111" s="13"/>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A112" s="12"/>
       <c r="E112" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="H112" s="13"/>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A113" s="12"/>
       <c r="E113" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="H113" s="13"/>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A114" s="12"/>
       <c r="E114" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="H114" s="13"/>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A115" s="12"/>
       <c r="E115" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="H115" s="13"/>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A116" s="12"/>
       <c r="E116" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="H116" s="13"/>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A117" s="12"/>
       <c r="E117" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="H117" s="13"/>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A118" s="12"/>
-      <c r="E118" t="s">
-        <v>182</v>
-      </c>
+      <c r="A118" s="14"/>
+      <c r="B118" s="15"/>
+      <c r="C118" s="16"/>
+      <c r="D118" s="16"/>
+      <c r="E118" s="16" t="s">
+        <v>186</v>
+      </c>
+      <c r="F118" s="16"/>
       <c r="H118" s="13"/>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A119" s="12"/>
       <c r="E119" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="H119" s="13"/>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A120" s="12"/>
       <c r="E120" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="H120" s="13"/>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A121" s="12"/>
       <c r="E121" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="H121" s="13"/>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A122" s="12"/>
       <c r="E122" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="H122" s="13"/>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A123" s="14"/>
-      <c r="B123" s="15"/>
-      <c r="C123" s="16"/>
-      <c r="D123" s="16"/>
-      <c r="E123" s="16" t="s">
-        <v>187</v>
-      </c>
-      <c r="F123" s="16"/>
+      <c r="E123" t="s">
+        <v>191</v>
+      </c>
       <c r="G123" s="16"/>
       <c r="H123" s="17"/>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E124" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E125" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E126" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E127" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E128" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="129" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E129" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="130" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E130" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="131" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E131" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="132" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E132" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
     <row r="133" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E133" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="134" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E134" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="135" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E135" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
     </row>
     <row r="136" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E136" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="137" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E137" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
     </row>
     <row r="138" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E138" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="139" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E139" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
     <row r="140" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E140" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="141" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E141" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="142" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E142" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="143" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E143" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="144" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E144" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="145" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E145" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="146" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E146" t="s">
         <v>210</v>
-      </c>
-    </row>
-    <row r="147" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E147" t="s">
-        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -2859,7 +3194,7 @@
   <sheetData>
     <row r="1" spans="1:5" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>0</v>
@@ -2885,68 +3220,68 @@
         <v>22</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B3" s="19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D3" s="18" t="s">
         <v>22</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="B4" s="19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>22</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B5" s="19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>22</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="B6" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D6" s="18" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="22" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -2959,31 +3294,978 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A417624D-655D-D64B-BD86-D9B240BEDD44}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.6640625" customWidth="1"/>
     <col min="2" max="2" width="17.6640625" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="5" max="5" width="24.1640625" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="17.5" customWidth="1"/>
+    <col min="6" max="6" width="27.33203125" customWidth="1"/>
+    <col min="7" max="7" width="21.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" s="10" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>212</v>
-      </c>
-      <c r="B1" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>214</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="26" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="26" t="s">
+        <v>216</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26" t="s">
+        <v>217</v>
+      </c>
+      <c r="H3" s="25" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="26" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>218</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>219</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>221</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B7" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>223</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>225</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>226</v>
+      </c>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26" t="s">
+        <v>227</v>
+      </c>
+      <c r="G8" s="25" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B9" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>228</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24" t="s">
+        <v>229</v>
+      </c>
+      <c r="G9" s="24" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B10" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>230</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B11" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>232</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B12" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>234</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B13" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>236</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B14" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>238</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B15" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>240</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B16" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>242</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="D17" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26" t="s">
+        <v>245</v>
+      </c>
+      <c r="G17" s="25" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="D18" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B19" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B20" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="C20" s="24" t="s">
+        <v>250</v>
+      </c>
+      <c r="D20" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B21" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>252</v>
+      </c>
+      <c r="D21" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B22" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="C22" s="24" t="s">
+        <v>254</v>
+      </c>
+      <c r="D22" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B23" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="C23" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="D23" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B24" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="C24" s="24" t="s">
+        <v>258</v>
+      </c>
+      <c r="D24" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="C25" s="27" t="s">
+        <v>260</v>
+      </c>
+      <c r="D25" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27" t="s">
+        <v>261</v>
+      </c>
+      <c r="G25" s="28" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="C26" s="27" t="s">
+        <v>262</v>
+      </c>
+      <c r="D26" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B27" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" s="24" t="s">
+        <v>264</v>
+      </c>
+      <c r="D27" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B28" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="C28" s="24" t="s">
+        <v>266</v>
+      </c>
+      <c r="D28" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B29" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29" s="24" t="s">
+        <v>268</v>
+      </c>
+      <c r="D29" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>270</v>
+      </c>
+      <c r="D30" s="27" t="s">
+        <v>226</v>
+      </c>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="C31" s="27" t="s">
+        <v>272</v>
+      </c>
+      <c r="D31" s="27" t="s">
+        <v>226</v>
+      </c>
+      <c r="E31" s="27"/>
+      <c r="F31" s="27" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B32" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="C32" s="24" t="s">
+        <v>274</v>
+      </c>
+      <c r="D32" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B33" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="C33" s="24" t="s">
+        <v>276</v>
+      </c>
+      <c r="D33" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B34" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="C34" s="24" t="s">
+        <v>278</v>
+      </c>
+      <c r="D34" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B35" s="24" t="s">
+        <v>131</v>
+      </c>
+      <c r="C35" s="24" t="s">
+        <v>280</v>
+      </c>
+      <c r="D35" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B36" s="24" t="s">
+        <v>132</v>
+      </c>
+      <c r="C36" s="24" t="s">
+        <v>282</v>
+      </c>
+      <c r="D36" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E36" s="24"/>
+      <c r="F36" s="24" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B37" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="C37" s="24" t="s">
+        <v>284</v>
+      </c>
+      <c r="D37" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B38" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="C38" s="24" t="s">
+        <v>286</v>
+      </c>
+      <c r="D38" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B39" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="C39" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="D39" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B40" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="C40" s="24" t="s">
+        <v>290</v>
+      </c>
+      <c r="D40" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E40" s="24"/>
+      <c r="F40" s="24" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B41" s="24" t="s">
+        <v>135</v>
+      </c>
+      <c r="C41" s="24" t="s">
+        <v>292</v>
+      </c>
+      <c r="D41" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E41" s="24"/>
+      <c r="F41" s="24" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B42" s="24" t="s">
+        <v>136</v>
+      </c>
+      <c r="C42" s="24" t="s">
+        <v>294</v>
+      </c>
+      <c r="D42" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E42" s="24"/>
+      <c r="F42" s="24" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B43" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="C43" s="24" t="s">
+        <v>296</v>
+      </c>
+      <c r="D43" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B44" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="C44" s="24" t="s">
+        <v>298</v>
+      </c>
+      <c r="D44" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B45" s="24" t="s">
+        <v>139</v>
+      </c>
+      <c r="C45" s="24" t="s">
+        <v>300</v>
+      </c>
+      <c r="D45" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E45" s="24"/>
+      <c r="F45" s="24" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B46" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="C46" s="24" t="s">
+        <v>302</v>
+      </c>
+      <c r="D46" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E46" s="24"/>
+      <c r="F46" s="24" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B47" s="24" t="s">
+        <v>141</v>
+      </c>
+      <c r="C47" s="24" t="s">
+        <v>304</v>
+      </c>
+      <c r="D47" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E47" s="24"/>
+      <c r="F47" s="24" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B48" s="24" t="s">
+        <v>142</v>
+      </c>
+      <c r="C48" s="24" t="s">
+        <v>306</v>
+      </c>
+      <c r="D48" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E48" s="24"/>
+      <c r="F48" s="24" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B49" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="C49" s="24" t="s">
+        <v>308</v>
+      </c>
+      <c r="D49" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E49" s="24"/>
+      <c r="F49" s="24" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B50" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="C50" s="24" t="s">
+        <v>310</v>
+      </c>
+      <c r="D50" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E50" s="24"/>
+      <c r="F50" s="24" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B51" s="24" t="s">
+        <v>145</v>
+      </c>
+      <c r="C51" s="24" t="s">
+        <v>312</v>
+      </c>
+      <c r="D51" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E51" s="24"/>
+      <c r="F51" s="24" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B52" s="24" t="s">
+        <v>146</v>
+      </c>
+      <c r="C52" s="24" t="s">
+        <v>314</v>
+      </c>
+      <c r="D52" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E52" s="24"/>
+      <c r="F52" s="24" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B53" s="24" t="s">
+        <v>147</v>
+      </c>
+      <c r="C53" s="24" t="s">
+        <v>316</v>
+      </c>
+      <c r="D53" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E53" s="24"/>
+      <c r="F53" s="24" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B54" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="C54" s="24" t="s">
+        <v>318</v>
+      </c>
+      <c r="D54" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E54" s="24"/>
+      <c r="F54" s="24" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B55" s="24" t="s">
+        <v>149</v>
+      </c>
+      <c r="C55" s="24" t="s">
+        <v>320</v>
+      </c>
+      <c r="D55" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E55" s="24"/>
+      <c r="F55" s="24" t="s">
+        <v>321</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{115DDB95-6503-3B46-8C84-E8ABEEF6693E}">
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.5" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="10" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="C1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="23" t="s">
         <v>6</v>
       </c>
+      <c r="F1" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="30" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="30" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="30" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B6" s="30" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="30" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="30" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B9" s="30" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B10" s="30" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B11" s="30" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B12" s="30" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B13" s="30" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B14" s="30" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B15" s="30" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="26" spans="9:9" x14ac:dyDescent="0.2">
+      <c r="I26" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
merging all the datasets, have not exported yet as cleaned data
</commit_message>
<xml_diff>
--- a/CleanData/DataDictionary.xlsx
+++ b/CleanData/DataDictionary.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ainsl/Desktop/R01_Aim1H1/CleanData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4CB20B5-BF20-AD43-A223-03198CFC2581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C0ED65-8F3F-1C42-B86B-AA98880D2C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16160" yWindow="920" windowWidth="13920" windowHeight="17580" activeTab="3" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
+    <workbookView xWindow="15680" yWindow="900" windowWidth="14400" windowHeight="17580" firstSheet="1" activeTab="2" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
   </bookViews>
   <sheets>
     <sheet name="CleanedData" sheetId="1" r:id="rId1"/>
     <sheet name="ALCUSE Data" sheetId="2" r:id="rId2"/>
     <sheet name="R6_2 Data" sheetId="3" r:id="rId3"/>
     <sheet name="SelfReported_DrinkingDriving" sheetId="4" r:id="rId4"/>
+    <sheet name="Primary Variables" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="332">
   <si>
     <t>Variable</t>
   </si>
@@ -396,18 +397,6 @@
     <t>Annual household income (in previous year)</t>
   </si>
   <si>
-    <t>poverty_cat</t>
-  </si>
-  <si>
-    <t>Poverty ratio</t>
-  </si>
-  <si>
-    <t>parent_edu_cat</t>
-  </si>
-  <si>
-    <t>Parent education</t>
-  </si>
-  <si>
     <t>employment_weeks_cat</t>
   </si>
   <si>
@@ -453,13 +442,7 @@
     <t>R1487800</t>
   </si>
   <si>
-    <t>S1541900</t>
-  </si>
-  <si>
     <t>S1225800</t>
-  </si>
-  <si>
-    <t>Combination of mom education (R1302700) and dad education (R1302600), taken at baseline</t>
   </si>
   <si>
     <t>R1235800</t>
@@ -1367,6 +1350,12 @@
     <t>physical_env_risk_num (and _cat)</t>
   </si>
   <si>
+    <t>dad_pmk (and dad_pmk_cat_</t>
+  </si>
+  <si>
+    <t>mom_pmk (and mom_pmk_cat)</t>
+  </si>
+  <si>
     <t>dad_style</t>
   </si>
   <si>
@@ -1385,12 +1374,6 @@
     <t>birthdate</t>
   </si>
   <si>
-    <t>mom_pmk_97 (and mom_pmk_97_cat)</t>
-  </si>
-  <si>
-    <t>dad_pmk_97 (and dad_pmk_97_cat_</t>
-  </si>
-  <si>
     <t>T1050200</t>
   </si>
   <si>
@@ -1410,6 +1393,72 @@
   </si>
   <si>
     <t>U2963200</t>
+  </si>
+  <si>
+    <t>Sex 1997</t>
+  </si>
+  <si>
+    <t>Duplicate from R6_2</t>
+  </si>
+  <si>
+    <t>Bdate M</t>
+  </si>
+  <si>
+    <t>Bdate Y</t>
+  </si>
+  <si>
+    <t>CV Sample Type</t>
+  </si>
+  <si>
+    <t>Race_ethnicity</t>
+  </si>
+  <si>
+    <t>Times reported drive when drinking 2002</t>
+  </si>
+  <si>
+    <t>1 = &gt;=1 time, 0 = no times</t>
+  </si>
+  <si>
+    <t>Same but for other years</t>
+  </si>
+  <si>
+    <t>""</t>
+  </si>
+  <si>
+    <t>Age at round 6</t>
+  </si>
+  <si>
+    <t>Primary</t>
+  </si>
+  <si>
+    <t>round6_weight file??</t>
+  </si>
+  <si>
+    <t>"Pre-21", "21-24"</t>
+  </si>
+  <si>
+    <t>SelfReported_DrinkingDriving</t>
+  </si>
+  <si>
+    <t>Binge Drinking</t>
+  </si>
+  <si>
+    <t>Marijuana use</t>
+  </si>
+  <si>
+    <t>" "</t>
+  </si>
+  <si>
+    <t>"0 TO 4", "5 TO 8", "9 TO 12", "13 TO 16"</t>
+  </si>
+  <si>
+    <t>???</t>
+  </si>
+  <si>
+    <t>Income in 2002 (past-year)</t>
+  </si>
+  <si>
+    <t>"No", "Yes"</t>
   </si>
 </sst>
 </file>
@@ -1499,7 +1548,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1521,6 +1570,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1640,7 +1695,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1722,6 +1777,17 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2063,7 +2129,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A5CC42-7E80-3145-82C3-AE1AB4759DCA}">
-  <dimension ref="A1:I127"/>
+  <dimension ref="A1:I125"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" customWidth="1"/>
@@ -2091,7 +2157,7 @@
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>34</v>
@@ -2111,7 +2177,7 @@
         <v>39</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="8" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.25">
@@ -2122,6 +2188,9 @@
       <c r="E3" s="8" t="s">
         <v>40</v>
       </c>
+      <c r="F3" s="8" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="4" spans="1:7" s="8" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -2131,6 +2200,9 @@
       <c r="E4" s="8" t="s">
         <v>42</v>
       </c>
+      <c r="F4" s="8" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="5" spans="1:7" s="10" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
@@ -2142,6 +2214,9 @@
       <c r="E5" s="7" t="s">
         <v>38</v>
       </c>
+      <c r="F5" s="7" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="6" spans="1:7" s="10" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
@@ -2156,6 +2231,9 @@
       <c r="E6" s="7" t="s">
         <v>53</v>
       </c>
+      <c r="F6" s="7" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="7" spans="1:7" s="10" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
@@ -2167,7 +2245,15 @@
       <c r="C7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="7"/>
+      <c r="D7" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="8" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -2185,13 +2271,19 @@
       <c r="E8" s="3" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="F8" s="3" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="42" customFormat="1" ht="68" x14ac:dyDescent="0.2">
+      <c r="A9" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="43" t="s">
         <v>10</v>
+      </c>
+      <c r="C9" s="42" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -2210,6 +2302,9 @@
       <c r="E10" t="s">
         <v>55</v>
       </c>
+      <c r="F10" s="3" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="11" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -2227,6 +2322,9 @@
       <c r="E11" t="s">
         <v>56</v>
       </c>
+      <c r="F11" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="12" spans="1:7" ht="170" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -2244,6 +2342,9 @@
       <c r="E12" t="s">
         <v>57</v>
       </c>
+      <c r="F12" t="s">
+        <v>275</v>
+      </c>
       <c r="G12" t="s">
         <v>35</v>
       </c>
@@ -2264,18 +2365,45 @@
       <c r="E13" t="s">
         <v>58</v>
       </c>
+      <c r="F13" t="s">
+        <v>275</v>
+      </c>
       <c r="G13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+        <v>271</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C14" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" t="s">
+        <v>328</v>
+      </c>
+      <c r="F14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>278</v>
+        <v>272</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C15" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" t="s">
+        <v>328</v>
+      </c>
+      <c r="F15" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="17" x14ac:dyDescent="0.2">
@@ -2294,6 +2422,9 @@
       <c r="E16" s="7" t="s">
         <v>59</v>
       </c>
+      <c r="F16" s="7" t="s">
+        <v>275</v>
+      </c>
       <c r="G16" t="s">
         <v>35</v>
       </c>
@@ -2311,6 +2442,9 @@
       <c r="E17" s="7" t="s">
         <v>60</v>
       </c>
+      <c r="F17" s="7" t="s">
+        <v>275</v>
+      </c>
       <c r="G17" t="s">
         <v>35</v>
       </c>
@@ -2328,6 +2462,9 @@
       <c r="E18" s="7" t="s">
         <v>61</v>
       </c>
+      <c r="F18" s="7" t="s">
+        <v>275</v>
+      </c>
       <c r="G18" t="s">
         <v>35</v>
       </c>
@@ -2348,6 +2485,9 @@
       <c r="E19" s="7" t="s">
         <v>64</v>
       </c>
+      <c r="F19" s="7" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="20" spans="1:9" ht="85" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
@@ -2363,7 +2503,10 @@
         <v>25</v>
       </c>
       <c r="E20" t="s">
-        <v>261</v>
+        <v>255</v>
+      </c>
+      <c r="F20" s="44" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -2373,12 +2516,18 @@
       <c r="B21" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
+      <c r="C21" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>331</v>
+      </c>
       <c r="E21" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="F21" s="18"/>
+        <v>81</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>275</v>
+      </c>
       <c r="G21" s="18" t="s">
         <v>43</v>
       </c>
@@ -2394,13 +2543,9 @@
       </c>
       <c r="C22" s="18"/>
       <c r="D22" s="18"/>
-      <c r="E22" s="18" t="s">
-        <v>85</v>
-      </c>
+      <c r="E22" s="18"/>
       <c r="F22" s="18"/>
-      <c r="G22" s="18" t="s">
-        <v>67</v>
-      </c>
+      <c r="G22" s="18"/>
       <c r="H22" s="18"/>
       <c r="I22" s="18"/>
     </row>
@@ -2413,220 +2558,210 @@
       </c>
       <c r="C23" s="18"/>
       <c r="D23" s="18"/>
-      <c r="E23" s="18" t="s">
-        <v>87</v>
-      </c>
+      <c r="E23" s="18"/>
       <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
+      <c r="G23" s="18" t="s">
+        <v>70</v>
+      </c>
       <c r="H23" s="18"/>
       <c r="I23" s="18"/>
     </row>
-    <row r="24" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="18" t="s">
-        <v>70</v>
+        <v>273</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
+        <v>274</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>275</v>
+      </c>
       <c r="G24" s="18"/>
       <c r="H24" s="18"/>
       <c r="I24" s="18"/>
     </row>
-    <row r="25" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A25" s="18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18" t="s">
-        <v>74</v>
-      </c>
+        <v>279</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>276</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>275</v>
+      </c>
+      <c r="G25" s="18"/>
       <c r="H25" s="18"/>
       <c r="I25" s="18"/>
     </row>
     <row r="26" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="18" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>287</v>
-      </c>
-      <c r="E26" s="18" t="s">
-        <v>82</v>
+        <v>282</v>
+      </c>
+      <c r="E26" s="26" t="s">
+        <v>77</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="G26" s="18"/>
       <c r="H26" s="18"/>
       <c r="I26" s="18"/>
     </row>
-    <row r="27" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="18" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="C27" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D27" s="19" t="s">
-        <v>282</v>
+      <c r="D27" s="18" t="s">
+        <v>283</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="G27" s="18"/>
       <c r="H27" s="18"/>
       <c r="I27" s="18"/>
     </row>
-    <row r="28" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="18" t="s">
-        <v>283</v>
+        <v>73</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>284</v>
-      </c>
-      <c r="C28" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="D28" s="18" t="s">
-        <v>288</v>
-      </c>
-      <c r="E28" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="F28" s="18" t="s">
-        <v>281</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="F28" s="18"/>
       <c r="G28" s="18"/>
       <c r="H28" s="18"/>
       <c r="I28" s="18"/>
     </row>
-    <row r="29" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="19" t="s">
-        <v>286</v>
-      </c>
       <c r="C29" s="18" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F29" s="18" t="s">
-        <v>281</v>
-      </c>
-      <c r="G29" s="18"/>
+        <v>275</v>
+      </c>
+      <c r="G29" s="18" t="s">
+        <v>291</v>
+      </c>
       <c r="H29" s="18"/>
       <c r="I29" s="18"/>
     </row>
-    <row r="30" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="B30" s="19" t="s">
-        <v>78</v>
-      </c>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
+        <v>285</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>286</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>287</v>
+      </c>
       <c r="E30" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="F30" s="18"/>
+        <v>127</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>275</v>
+      </c>
       <c r="G30" s="18"/>
       <c r="H30" s="18"/>
       <c r="I30" s="18"/>
     </row>
-    <row r="31" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A31" s="18" t="s">
-        <v>79</v>
+        <v>288</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="C31" s="18" t="s">
-        <v>21</v>
-      </c>
+        <v>290</v>
+      </c>
+      <c r="C31" s="18"/>
       <c r="D31" s="18" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>84</v>
+        <v>129</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>281</v>
-      </c>
-      <c r="G31" s="18" t="s">
-        <v>297</v>
-      </c>
+        <v>275</v>
+      </c>
+      <c r="G31" s="18"/>
       <c r="H31" s="18"/>
       <c r="I31" s="18"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A32" s="18" t="s">
-        <v>291</v>
-      </c>
-      <c r="B32" s="18" t="s">
-        <v>292</v>
-      </c>
-      <c r="C32" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="D32" s="18" t="s">
-        <v>293</v>
-      </c>
-      <c r="E32" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="F32" s="18" t="s">
-        <v>281</v>
-      </c>
+      <c r="A32" s="18"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
       <c r="G32" s="18"/>
       <c r="H32" s="18"/>
       <c r="I32" s="18"/>
     </row>
-    <row r="33" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A33" s="18" t="s">
-        <v>294</v>
-      </c>
-      <c r="B33" s="19" t="s">
-        <v>296</v>
-      </c>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A33" s="18"/>
+      <c r="B33" s="19"/>
       <c r="C33" s="18"/>
-      <c r="D33" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="E33" s="18" t="s">
-        <v>135</v>
-      </c>
-      <c r="F33" s="18" t="s">
-        <v>281</v>
-      </c>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
       <c r="G33" s="18"/>
       <c r="H33" s="18"/>
       <c r="I33" s="18"/>
@@ -2819,30 +2954,20 @@
       <c r="I50" s="18"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A51" s="18"/>
-      <c r="B51" s="19"/>
-      <c r="C51" s="18"/>
-      <c r="D51" s="18"/>
-      <c r="E51" s="18"/>
-      <c r="F51" s="18"/>
+      <c r="A51" s="12"/>
+      <c r="E51" s="20"/>
       <c r="G51" s="18"/>
       <c r="H51" s="18"/>
       <c r="I51" s="18"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A52" s="18"/>
-      <c r="B52" s="19"/>
-      <c r="C52" s="18"/>
-      <c r="D52" s="18"/>
-      <c r="E52" s="18"/>
-      <c r="F52" s="18"/>
+      <c r="A52" s="12"/>
       <c r="G52" s="18"/>
       <c r="H52" s="18"/>
       <c r="I52" s="18"/>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" s="12"/>
-      <c r="E53" s="20"/>
       <c r="G53" s="18"/>
       <c r="H53" s="18"/>
       <c r="I53" s="18"/>
@@ -2861,15 +2986,11 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" s="12"/>
-      <c r="G56" s="18"/>
-      <c r="H56" s="18"/>
-      <c r="I56" s="18"/>
+      <c r="H56" s="13"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" s="12"/>
-      <c r="G57" s="18"/>
-      <c r="H57" s="18"/>
-      <c r="I57" s="18"/>
+      <c r="H57" s="13"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="12"/>
@@ -3120,20 +3241,18 @@
       <c r="H119" s="13"/>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A120" s="12"/>
+      <c r="A120" s="14"/>
+      <c r="B120" s="15"/>
+      <c r="C120" s="16"/>
+      <c r="D120" s="16"/>
+      <c r="E120" s="16"/>
+      <c r="F120" s="16"/>
       <c r="H120" s="13"/>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A121" s="12"/>
       <c r="H121" s="13"/>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A122" s="14"/>
-      <c r="B122" s="15"/>
-      <c r="C122" s="16"/>
-      <c r="D122" s="16"/>
-      <c r="E122" s="16"/>
-      <c r="F122" s="16"/>
       <c r="H122" s="13"/>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.2">
@@ -3143,14 +3262,8 @@
       <c r="H124" s="13"/>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H125" s="13"/>
-    </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H126" s="13"/>
-    </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="G127" s="16"/>
-      <c r="H127" s="17"/>
+      <c r="G125" s="16"/>
+      <c r="H125" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3170,7 +3283,7 @@
   <sheetData>
     <row r="1" spans="1:6" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>0</v>
@@ -3190,90 +3303,90 @@
     </row>
     <row r="2" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="D2" s="18" t="s">
         <v>21</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="D3" s="18" t="s">
         <v>21</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>21</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>21</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="F5" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="D6" s="18" t="s">
         <v>21</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3289,7 +3402,7 @@
     </row>
     <row r="11" spans="1:6" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="31" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -3302,7 +3415,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A417624D-655D-D64B-BD86-D9B240BEDD44}">
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.6640625" customWidth="1"/>
@@ -3316,7 +3429,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="10" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>2</v>
@@ -3357,881 +3470,897 @@
         <v>59</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D3" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E3" s="33" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="24" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="D4" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E4" s="34"/>
       <c r="F4" s="25" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="H4" s="24" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="24" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="D5" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E5" s="34"/>
       <c r="F5" s="25" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="24" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="24" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B6" s="25" t="s">
         <v>61</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D6" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="F6" s="25" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="24" customFormat="1" ht="112" x14ac:dyDescent="0.2">
       <c r="A7" s="24" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="B7" s="25" t="s">
         <v>60</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D7" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B8" s="23" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="D8" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E8" s="35"/>
       <c r="F8" s="23" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B9" s="25" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E9" s="34"/>
       <c r="F9" s="25" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B10" s="23" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E10" s="35"/>
       <c r="F10" s="23" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B11" s="23" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E11" s="35"/>
       <c r="F11" s="23" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B12" s="23" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D12" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E12" s="35"/>
       <c r="F12" s="23" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B13" s="23" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="D13" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E13" s="35"/>
       <c r="F13" s="23" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B14" s="23" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="D14" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="35"/>
       <c r="F14" s="23" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B15" s="23" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D15" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E15" s="35"/>
       <c r="F15" s="23" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B16" s="23" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D16" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E16" s="35"/>
       <c r="F16" s="23" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="24" customFormat="1" ht="80" x14ac:dyDescent="0.2">
       <c r="A17" s="24" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D17" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="F17" s="25" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="18" spans="1:7" s="24" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="B18" s="25" t="s">
         <v>58</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D18" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="F18" s="25" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="24" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A19" s="27" t="s">
-        <v>308</v>
+        <v>295</v>
       </c>
       <c r="B19" s="25" t="s">
         <v>57</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D19" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E19" s="34" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="F19" s="25" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B20" s="23" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D20" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E20" s="35"/>
       <c r="F20" s="23" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B21" s="23" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="D21" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E21" s="35"/>
       <c r="F21" s="23" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B22" s="23" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="D22" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E22" s="35"/>
       <c r="F22" s="23" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B23" s="23" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="D23" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E23" s="35"/>
       <c r="F23" s="23" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B24" s="23" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D24" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E24" s="35"/>
       <c r="F24" s="23" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B25" s="23" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="D25" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E25" s="35"/>
       <c r="F25" s="23" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
     </row>
     <row r="26" spans="1:7" s="27" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="D26" s="26" t="s">
         <v>27</v>
       </c>
       <c r="E26" s="36" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="F26" s="26" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="G26" s="27" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="27" spans="1:7" s="27" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A27" s="27" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="D27" s="26" t="s">
         <v>27</v>
       </c>
       <c r="E27" s="36" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="F27" s="26" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B28" s="23" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="D28" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E28" s="35"/>
       <c r="F28" s="23" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B29" s="23" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="D29" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E29" s="35"/>
       <c r="F29" s="23" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B30" s="23" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="D30" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E30" s="35"/>
       <c r="F30" s="23" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="31" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="18" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="D31" s="26" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E31" s="36"/>
       <c r="F31" s="26" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="32" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="27" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="D32" s="26" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E32" s="36"/>
       <c r="F32" s="26" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B33" s="23" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E33" s="35"/>
       <c r="F33" s="23" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B34" s="23" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="D34" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E34" s="35"/>
       <c r="F34" s="23" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B35" s="23" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="D35" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E35" s="35"/>
       <c r="F35" s="23" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B36" s="23" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="D36" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E36" s="35"/>
       <c r="F36" s="23" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B37" s="23" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="D37" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E37" s="35"/>
       <c r="F37" s="23" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B38" s="23" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E38" s="35"/>
       <c r="F38" s="23" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
     </row>
     <row r="39" spans="1:6" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="24" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B39" s="25" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C39" s="25" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="D39" s="25" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E39" s="34"/>
       <c r="F39" s="25" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B40" s="23" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="D40" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E40" s="35"/>
       <c r="F40" s="23" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B41" s="23" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="D41" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E41" s="35"/>
       <c r="F41" s="23" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B42" s="23" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="D42" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E42" s="35"/>
       <c r="F42" s="23" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B43" s="23" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E43" s="35"/>
       <c r="F43" s="23" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
     </row>
     <row r="44" spans="1:6" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="24" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="B44" s="25" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C44" s="25" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="D44" s="25" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E44" s="34"/>
       <c r="F44" s="25" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B45" s="23" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="D45" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E45" s="35"/>
       <c r="F45" s="23" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
     </row>
     <row r="46" spans="1:6" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="24" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="B46" s="25" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="C46" s="25" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="D46" s="25" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E46" s="34"/>
       <c r="F46" s="25" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B47" s="23" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="D47" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E47" s="35"/>
       <c r="F47" s="23" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B48" s="23" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E48" s="35"/>
       <c r="F48" s="23" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.2">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B49" s="23" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E49" s="35"/>
       <c r="F49" s="23" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.2">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B50" s="23" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="D50" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E50" s="35"/>
       <c r="F50" s="23" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.2">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B51" s="23" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E51" s="35"/>
       <c r="F51" s="23" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.2">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B52" s="23" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C52" s="23" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E52" s="35"/>
       <c r="F52" s="23" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.2">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B53" s="23" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C53" s="23" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E53" s="35"/>
       <c r="F53" s="23" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.2">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B54" s="23" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C54" s="23" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E54" s="35"/>
       <c r="F54" s="23" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.2">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B55" s="23" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C55" s="23" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="D55" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E55" s="35"/>
       <c r="F55" s="23" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.2">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B56" s="23" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C56" s="23" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E56" s="35"/>
       <c r="F56" s="23" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>62</v>
+      </c>
+      <c r="B57" s="23" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>23</v>
+      </c>
+      <c r="B58" t="s">
         <v>255</v>
       </c>
     </row>
@@ -4248,13 +4377,15 @@
     <col min="1" max="1" width="15.5" customWidth="1"/>
     <col min="2" max="2" width="14.33203125" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="18.5" customWidth="1"/>
     <col min="5" max="5" width="19.33203125" customWidth="1"/>
     <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="25.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="10" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>2</v>
@@ -4277,82 +4408,271 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="B2" t="s">
         <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B3" s="29" t="s">
         <v>59</v>
       </c>
+      <c r="C3" t="s">
+        <v>310</v>
+      </c>
+      <c r="G3" t="s">
+        <v>311</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B4" s="29" t="s">
-        <v>102</v>
+        <v>96</v>
+      </c>
+      <c r="C4" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B5" s="29" t="s">
-        <v>103</v>
+        <v>97</v>
+      </c>
+      <c r="C5" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B6" s="29" t="s">
-        <v>88</v>
+        <v>82</v>
+      </c>
+      <c r="C6" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B7" s="29" t="s">
-        <v>112</v>
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
       <c r="B8" s="29" t="s">
         <v>54</v>
       </c>
+      <c r="C8" t="s">
+        <v>316</v>
+      </c>
+      <c r="E8" t="s">
+        <v>317</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B9" s="29" t="s">
-        <v>309</v>
+        <v>303</v>
+      </c>
+      <c r="C9" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B10" s="29" t="s">
-        <v>310</v>
+        <v>304</v>
+      </c>
+      <c r="C10" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B11" s="29" t="s">
-        <v>311</v>
+        <v>305</v>
+      </c>
+      <c r="C11" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B12" s="29" t="s">
-        <v>312</v>
+        <v>306</v>
+      </c>
+      <c r="C12" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B13" s="29" t="s">
-        <v>313</v>
+        <v>307</v>
+      </c>
+      <c r="C13" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B14" s="29" t="s">
-        <v>314</v>
+        <v>308</v>
+      </c>
+      <c r="C14" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B15" s="29" t="s">
-        <v>315</v>
+        <v>309</v>
+      </c>
+      <c r="C15" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="26" spans="9:9" x14ac:dyDescent="0.2">
       <c r="I26" s="28"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B7A2A69-B0C6-1A43-B3A0-CA6A06B448A8}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.6640625" customWidth="1"/>
+    <col min="7" max="7" width="29.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="10" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+      <c r="A3" s="40" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="41" t="s">
+        <v>325</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" s="40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="41" t="s">
+        <v>320</v>
+      </c>
+      <c r="D4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="41" t="s">
+        <v>326</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="128" x14ac:dyDescent="0.2">
+      <c r="A6" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>42</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
adding pmk from other years
</commit_message>
<xml_diff>
--- a/CleanData/DataDictionary.xlsx
+++ b/CleanData/DataDictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ainsl/Desktop/R01_Aim1H1/CleanData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C0ED65-8F3F-1C42-B86B-AA98880D2C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C99A14B-3B99-3B45-8579-F9FABA42192C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15680" yWindow="900" windowWidth="14400" windowHeight="17580" firstSheet="1" activeTab="2" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
   </bookViews>
   <sheets>
     <sheet name="CleanedData" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="326">
   <si>
     <t>Variable</t>
   </si>
@@ -397,21 +397,6 @@
     <t>Annual household income (in previous year)</t>
   </si>
   <si>
-    <t>employment_weeks_cat</t>
-  </si>
-  <si>
-    <t>Weeks employed in 2002</t>
-  </si>
-  <si>
-    <t>parent_monitoring_cat</t>
-  </si>
-  <si>
-    <t>Parental monitoring</t>
-  </si>
-  <si>
-    <t>Combination of mom and dad?? Perhaps should take an average instead, in case of one parent household??</t>
-  </si>
-  <si>
     <t>family_home_risk_cat</t>
   </si>
   <si>
@@ -1429,9 +1414,6 @@
   </si>
   <si>
     <t>Primary</t>
-  </si>
-  <si>
-    <t>round6_weight file??</t>
   </si>
   <si>
     <t>"Pre-21", "21-24"</t>
@@ -2129,12 +2111,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A5CC42-7E80-3145-82C3-AE1AB4759DCA}">
-  <dimension ref="A1:I125"/>
+  <dimension ref="A1:I123"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" customWidth="1"/>
     <col min="2" max="2" width="21.1640625" style="2" customWidth="1"/>
-    <col min="3" max="4" width="21.1640625" customWidth="1"/>
+    <col min="3" max="3" width="21.1640625" customWidth="1"/>
+    <col min="4" max="4" width="21.1640625" style="2" customWidth="1"/>
     <col min="5" max="5" width="19.1640625" customWidth="1"/>
     <col min="6" max="6" width="27.6640625" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
@@ -2150,14 +2133,14 @@
       <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>34</v>
@@ -2173,11 +2156,12 @@
       <c r="C2" s="7" t="s">
         <v>27</v>
       </c>
+      <c r="D2" s="3"/>
       <c r="E2" s="7" t="s">
         <v>39</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="8" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.25">
@@ -2185,11 +2169,12 @@
         <v>33</v>
       </c>
       <c r="B3" s="9"/>
+      <c r="D3" s="9"/>
       <c r="E3" s="8" t="s">
         <v>40</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="8" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.25">
@@ -2197,11 +2182,12 @@
         <v>41</v>
       </c>
       <c r="B4" s="9"/>
+      <c r="D4" s="9"/>
       <c r="E4" s="8" t="s">
         <v>42</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="10" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.2">
@@ -2211,11 +2197,15 @@
       <c r="B5" s="3" t="s">
         <v>37</v>
       </c>
+      <c r="C5" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="21"/>
       <c r="E5" s="7" t="s">
         <v>38</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>322</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="10" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.2">
@@ -2228,11 +2218,12 @@
       <c r="C6" s="7" t="s">
         <v>46</v>
       </c>
+      <c r="D6" s="21"/>
       <c r="E6" s="7" t="s">
         <v>53</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="10" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.2">
@@ -2245,14 +2236,14 @@
       <c r="C7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>323</v>
+      <c r="D7" s="21" t="s">
+        <v>317</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>53</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -2272,7 +2263,7 @@
         <v>54</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="42" customFormat="1" ht="68" x14ac:dyDescent="0.2">
@@ -2283,8 +2274,9 @@
         <v>10</v>
       </c>
       <c r="C9" s="42" t="s">
-        <v>329</v>
-      </c>
+        <v>323</v>
+      </c>
+      <c r="D9" s="43"/>
     </row>
     <row r="10" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -2303,7 +2295,7 @@
         <v>55</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2323,7 +2315,7 @@
         <v>56</v>
       </c>
       <c r="F11" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="170" x14ac:dyDescent="0.2">
@@ -2336,14 +2328,14 @@
       <c r="C12" t="s">
         <v>46</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="2" t="s">
         <v>16</v>
       </c>
       <c r="E12" t="s">
         <v>57</v>
       </c>
       <c r="F12" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="G12" t="s">
         <v>35</v>
@@ -2359,54 +2351,54 @@
       <c r="C13" t="s">
         <v>46</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="2" t="s">
         <v>16</v>
       </c>
       <c r="E13" t="s">
         <v>58</v>
       </c>
       <c r="F13" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="G13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="C14" t="s">
         <v>27</v>
       </c>
-      <c r="D14" t="s">
-        <v>328</v>
+      <c r="D14" s="2" t="s">
+        <v>322</v>
       </c>
       <c r="F14" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="C15" t="s">
         <v>27</v>
       </c>
-      <c r="D15" t="s">
-        <v>328</v>
+      <c r="D15" s="2" t="s">
+        <v>322</v>
       </c>
       <c r="F15" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -2416,14 +2408,14 @@
       <c r="C16" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="3" t="s">
         <v>28</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>59</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="G16" t="s">
         <v>35</v>
@@ -2443,7 +2435,7 @@
         <v>60</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="G17" t="s">
         <v>35</v>
@@ -2463,7 +2455,7 @@
         <v>61</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="G18" t="s">
         <v>35</v>
@@ -2486,7 +2478,7 @@
         <v>64</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="85" x14ac:dyDescent="0.2">
@@ -2503,10 +2495,10 @@
         <v>25</v>
       </c>
       <c r="E20" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="F20" s="44" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -2519,14 +2511,14 @@
       <c r="C21" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D21" s="18" t="s">
-        <v>331</v>
+      <c r="D21" s="19" t="s">
+        <v>325</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="G21" s="18" t="s">
         <v>43</v>
@@ -2534,212 +2526,202 @@
       <c r="H21" s="18"/>
       <c r="I21" s="18"/>
     </row>
-    <row r="22" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="18" t="s">
-        <v>66</v>
+        <v>268</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
+        <v>269</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>276</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>270</v>
+      </c>
       <c r="G22" s="18"/>
       <c r="H22" s="18"/>
       <c r="I22" s="18"/>
     </row>
-    <row r="23" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A23" s="18" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18" t="s">
-        <v>70</v>
-      </c>
+        <v>274</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>271</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="G23" s="18"/>
       <c r="H23" s="18"/>
       <c r="I23" s="18"/>
     </row>
     <row r="24" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="18" t="s">
+        <v>272</v>
+      </c>
+      <c r="B24" s="19" t="s">
         <v>273</v>
       </c>
-      <c r="B24" s="19" t="s">
-        <v>274</v>
-      </c>
       <c r="C24" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="D24" s="18" t="s">
-        <v>281</v>
-      </c>
-      <c r="E24" s="18" t="s">
-        <v>78</v>
+        <v>149</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>277</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>72</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="G24" s="18"/>
       <c r="H24" s="18"/>
       <c r="I24" s="18"/>
     </row>
-    <row r="25" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="18" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="C25" s="18" t="s">
         <v>27</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="G25" s="18"/>
       <c r="H25" s="18"/>
       <c r="I25" s="18"/>
     </row>
-    <row r="26" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" s="18" t="s">
-        <v>277</v>
+        <v>68</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>278</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="D26" s="18" t="s">
-        <v>282</v>
-      </c>
-      <c r="E26" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="F26" s="18" t="s">
-        <v>275</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="C26" s="18"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="F26" s="18"/>
       <c r="G26" s="18"/>
       <c r="H26" s="18"/>
       <c r="I26" s="18"/>
     </row>
     <row r="27" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="18" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>280</v>
+        <v>71</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D27" s="18" t="s">
-        <v>283</v>
+        <v>21</v>
+      </c>
+      <c r="D27" s="19" t="s">
+        <v>279</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>275</v>
-      </c>
-      <c r="G27" s="18"/>
+        <v>270</v>
+      </c>
+      <c r="G27" s="18" t="s">
+        <v>286</v>
+      </c>
       <c r="H27" s="18"/>
       <c r="I27" s="18"/>
     </row>
     <row r="28" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="B28" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
+        <v>280</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>282</v>
+      </c>
       <c r="E28" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="F28" s="18"/>
+        <v>122</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>270</v>
+      </c>
       <c r="G28" s="18"/>
       <c r="H28" s="18"/>
       <c r="I28" s="18"/>
     </row>
-    <row r="29" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A29" s="18" t="s">
-        <v>75</v>
+        <v>283</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="C29" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D29" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="C29" s="18"/>
+      <c r="D29" s="19" t="s">
         <v>284</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>80</v>
+        <v>124</v>
       </c>
       <c r="F29" s="18" t="s">
-        <v>275</v>
-      </c>
-      <c r="G29" s="18" t="s">
-        <v>291</v>
-      </c>
+        <v>270</v>
+      </c>
+      <c r="G29" s="18"/>
       <c r="H29" s="18"/>
       <c r="I29" s="18"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A30" s="18" t="s">
-        <v>285</v>
-      </c>
-      <c r="B30" s="18" t="s">
-        <v>286</v>
-      </c>
-      <c r="C30" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="D30" s="18" t="s">
-        <v>287</v>
-      </c>
-      <c r="E30" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="F30" s="18" t="s">
-        <v>275</v>
-      </c>
+      <c r="A30" s="18"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
       <c r="G30" s="18"/>
       <c r="H30" s="18"/>
       <c r="I30" s="18"/>
     </row>
-    <row r="31" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A31" s="18" t="s">
-        <v>288</v>
-      </c>
-      <c r="B31" s="19" t="s">
-        <v>290</v>
-      </c>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" s="18"/>
+      <c r="B31" s="19"/>
       <c r="C31" s="18"/>
-      <c r="D31" s="18" t="s">
-        <v>289</v>
-      </c>
-      <c r="E31" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="F31" s="18" t="s">
-        <v>275</v>
-      </c>
+      <c r="D31" s="19"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="18"/>
       <c r="G31" s="18"/>
       <c r="H31" s="18"/>
       <c r="I31" s="18"/>
@@ -2748,7 +2730,7 @@
       <c r="A32" s="18"/>
       <c r="B32" s="19"/>
       <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
+      <c r="D32" s="19"/>
       <c r="E32" s="18"/>
       <c r="F32" s="18"/>
       <c r="G32" s="18"/>
@@ -2759,7 +2741,7 @@
       <c r="A33" s="18"/>
       <c r="B33" s="19"/>
       <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
+      <c r="D33" s="19"/>
       <c r="E33" s="18"/>
       <c r="F33" s="18"/>
       <c r="G33" s="18"/>
@@ -2770,7 +2752,7 @@
       <c r="A34" s="18"/>
       <c r="B34" s="19"/>
       <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
+      <c r="D34" s="19"/>
       <c r="E34" s="18"/>
       <c r="F34" s="18"/>
       <c r="G34" s="18"/>
@@ -2781,7 +2763,7 @@
       <c r="A35" s="18"/>
       <c r="B35" s="19"/>
       <c r="C35" s="18"/>
-      <c r="D35" s="18"/>
+      <c r="D35" s="19"/>
       <c r="E35" s="18"/>
       <c r="F35" s="18"/>
       <c r="G35" s="18"/>
@@ -2792,7 +2774,7 @@
       <c r="A36" s="18"/>
       <c r="B36" s="19"/>
       <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
+      <c r="D36" s="19"/>
       <c r="E36" s="18"/>
       <c r="F36" s="18"/>
       <c r="G36" s="18"/>
@@ -2803,7 +2785,7 @@
       <c r="A37" s="18"/>
       <c r="B37" s="19"/>
       <c r="C37" s="18"/>
-      <c r="D37" s="18"/>
+      <c r="D37" s="19"/>
       <c r="E37" s="18"/>
       <c r="F37" s="18"/>
       <c r="G37" s="18"/>
@@ -2814,7 +2796,7 @@
       <c r="A38" s="18"/>
       <c r="B38" s="19"/>
       <c r="C38" s="18"/>
-      <c r="D38" s="18"/>
+      <c r="D38" s="19"/>
       <c r="E38" s="18"/>
       <c r="F38" s="18"/>
       <c r="G38" s="18"/>
@@ -2825,7 +2807,7 @@
       <c r="A39" s="18"/>
       <c r="B39" s="19"/>
       <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
+      <c r="D39" s="19"/>
       <c r="E39" s="18"/>
       <c r="F39" s="18"/>
       <c r="G39" s="18"/>
@@ -2836,7 +2818,7 @@
       <c r="A40" s="18"/>
       <c r="B40" s="19"/>
       <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
+      <c r="D40" s="19"/>
       <c r="E40" s="18"/>
       <c r="F40" s="18"/>
       <c r="G40" s="18"/>
@@ -2847,7 +2829,7 @@
       <c r="A41" s="18"/>
       <c r="B41" s="19"/>
       <c r="C41" s="18"/>
-      <c r="D41" s="18"/>
+      <c r="D41" s="19"/>
       <c r="E41" s="18"/>
       <c r="F41" s="18"/>
       <c r="G41" s="18"/>
@@ -2858,7 +2840,7 @@
       <c r="A42" s="18"/>
       <c r="B42" s="19"/>
       <c r="C42" s="18"/>
-      <c r="D42" s="18"/>
+      <c r="D42" s="19"/>
       <c r="E42" s="18"/>
       <c r="F42" s="18"/>
       <c r="G42" s="18"/>
@@ -2869,7 +2851,7 @@
       <c r="A43" s="18"/>
       <c r="B43" s="19"/>
       <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
+      <c r="D43" s="19"/>
       <c r="E43" s="18"/>
       <c r="F43" s="18"/>
       <c r="G43" s="18"/>
@@ -2880,7 +2862,7 @@
       <c r="A44" s="18"/>
       <c r="B44" s="19"/>
       <c r="C44" s="18"/>
-      <c r="D44" s="18"/>
+      <c r="D44" s="19"/>
       <c r="E44" s="18"/>
       <c r="F44" s="18"/>
       <c r="G44" s="18"/>
@@ -2891,7 +2873,7 @@
       <c r="A45" s="18"/>
       <c r="B45" s="19"/>
       <c r="C45" s="18"/>
-      <c r="D45" s="18"/>
+      <c r="D45" s="19"/>
       <c r="E45" s="18"/>
       <c r="F45" s="18"/>
       <c r="G45" s="18"/>
@@ -2902,7 +2884,7 @@
       <c r="A46" s="18"/>
       <c r="B46" s="19"/>
       <c r="C46" s="18"/>
-      <c r="D46" s="18"/>
+      <c r="D46" s="19"/>
       <c r="E46" s="18"/>
       <c r="F46" s="18"/>
       <c r="G46" s="18"/>
@@ -2913,7 +2895,7 @@
       <c r="A47" s="18"/>
       <c r="B47" s="19"/>
       <c r="C47" s="18"/>
-      <c r="D47" s="18"/>
+      <c r="D47" s="19"/>
       <c r="E47" s="18"/>
       <c r="F47" s="18"/>
       <c r="G47" s="18"/>
@@ -2924,7 +2906,7 @@
       <c r="A48" s="18"/>
       <c r="B48" s="19"/>
       <c r="C48" s="18"/>
-      <c r="D48" s="18"/>
+      <c r="D48" s="19"/>
       <c r="E48" s="18"/>
       <c r="F48" s="18"/>
       <c r="G48" s="18"/>
@@ -2932,30 +2914,20 @@
       <c r="I48" s="18"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A49" s="18"/>
-      <c r="B49" s="19"/>
-      <c r="C49" s="18"/>
-      <c r="D49" s="18"/>
-      <c r="E49" s="18"/>
-      <c r="F49" s="18"/>
+      <c r="A49" s="12"/>
+      <c r="E49" s="20"/>
       <c r="G49" s="18"/>
       <c r="H49" s="18"/>
       <c r="I49" s="18"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A50" s="18"/>
-      <c r="B50" s="19"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="18"/>
-      <c r="E50" s="18"/>
-      <c r="F50" s="18"/>
+      <c r="A50" s="12"/>
       <c r="G50" s="18"/>
       <c r="H50" s="18"/>
       <c r="I50" s="18"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="12"/>
-      <c r="E51" s="20"/>
       <c r="G51" s="18"/>
       <c r="H51" s="18"/>
       <c r="I51" s="18"/>
@@ -2974,15 +2946,11 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" s="12"/>
-      <c r="G54" s="18"/>
-      <c r="H54" s="18"/>
-      <c r="I54" s="18"/>
+      <c r="H54" s="13"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" s="12"/>
-      <c r="G55" s="18"/>
-      <c r="H55" s="18"/>
-      <c r="I55" s="18"/>
+      <c r="H55" s="13"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" s="12"/>
@@ -3233,20 +3201,18 @@
       <c r="H117" s="13"/>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A118" s="12"/>
+      <c r="A118" s="14"/>
+      <c r="B118" s="15"/>
+      <c r="C118" s="16"/>
+      <c r="D118" s="15"/>
+      <c r="E118" s="16"/>
+      <c r="F118" s="16"/>
       <c r="H118" s="13"/>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A119" s="12"/>
       <c r="H119" s="13"/>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A120" s="14"/>
-      <c r="B120" s="15"/>
-      <c r="C120" s="16"/>
-      <c r="D120" s="16"/>
-      <c r="E120" s="16"/>
-      <c r="F120" s="16"/>
       <c r="H120" s="13"/>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.2">
@@ -3256,14 +3222,8 @@
       <c r="H122" s="13"/>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H123" s="13"/>
-    </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H124" s="13"/>
-    </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="G125" s="16"/>
-      <c r="H125" s="17"/>
+      <c r="G123" s="16"/>
+      <c r="H123" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3283,7 +3243,7 @@
   <sheetData>
     <row r="1" spans="1:6" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>0</v>
@@ -3303,90 +3263,90 @@
     </row>
     <row r="2" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D2" s="18" t="s">
         <v>21</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D3" s="18" t="s">
         <v>21</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>21</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>21</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F5" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D6" s="18" t="s">
         <v>21</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3402,7 +3362,7 @@
     </row>
     <row r="11" spans="1:6" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="31" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -3429,7 +3389,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="10" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>2</v>
@@ -3470,882 +3430,882 @@
         <v>59</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D3" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E3" s="33" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="24" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D4" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E4" s="34"/>
       <c r="F4" s="25" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="H4" s="24" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="24" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D5" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E5" s="34"/>
       <c r="F5" s="25" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="24" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="24" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="B6" s="25" t="s">
         <v>61</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D6" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="F6" s="25" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="24" customFormat="1" ht="112" x14ac:dyDescent="0.2">
       <c r="A7" s="24" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="B7" s="25" t="s">
         <v>60</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D7" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B8" s="23" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D8" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E8" s="35"/>
       <c r="F8" s="23" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B9" s="25" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E9" s="34"/>
       <c r="F9" s="25" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B10" s="23" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E10" s="35"/>
       <c r="F10" s="23" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B11" s="23" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E11" s="35"/>
       <c r="F11" s="23" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B12" s="23" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D12" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E12" s="35"/>
       <c r="F12" s="23" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B13" s="23" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="D13" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E13" s="35"/>
       <c r="F13" s="23" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B14" s="23" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="D14" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="35"/>
       <c r="F14" s="23" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B15" s="23" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D15" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E15" s="35"/>
       <c r="F15" s="23" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B16" s="23" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="D16" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E16" s="35"/>
       <c r="F16" s="23" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="24" customFormat="1" ht="80" x14ac:dyDescent="0.2">
       <c r="A17" s="24" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="D17" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="F17" s="25" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18" spans="1:7" s="24" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B18" s="25" t="s">
         <v>58</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="D18" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="F18" s="25" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="24" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A19" s="27" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="B19" s="25" t="s">
         <v>57</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="D19" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E19" s="34" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="F19" s="25" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B20" s="23" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="D20" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E20" s="35"/>
       <c r="F20" s="23" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B21" s="23" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="D21" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E21" s="35"/>
       <c r="F21" s="23" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B22" s="23" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="D22" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E22" s="35"/>
       <c r="F22" s="23" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B23" s="23" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="D23" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E23" s="35"/>
       <c r="F23" s="23" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B24" s="23" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="D24" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E24" s="35"/>
       <c r="F24" s="23" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B25" s="23" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="D25" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E25" s="35"/>
       <c r="F25" s="23" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="26" spans="1:7" s="27" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="D26" s="26" t="s">
         <v>27</v>
       </c>
       <c r="E26" s="36" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="F26" s="26" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="G26" s="27" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
     </row>
     <row r="27" spans="1:7" s="27" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A27" s="27" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="D27" s="26" t="s">
         <v>27</v>
       </c>
       <c r="E27" s="36" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="F27" s="26" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B28" s="23" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="D28" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E28" s="35"/>
       <c r="F28" s="23" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B29" s="23" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="D29" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E29" s="35"/>
       <c r="F29" s="23" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B30" s="23" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D30" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E30" s="35"/>
       <c r="F30" s="23" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="31" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="18" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="D31" s="26" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E31" s="36"/>
       <c r="F31" s="26" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="32" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="27" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="D32" s="26" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E32" s="36"/>
       <c r="F32" s="26" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B33" s="23" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E33" s="35"/>
       <c r="F33" s="23" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B34" s="23" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="D34" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E34" s="35"/>
       <c r="F34" s="23" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B35" s="23" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D35" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E35" s="35"/>
       <c r="F35" s="23" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B36" s="23" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="D36" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E36" s="35"/>
       <c r="F36" s="23" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B37" s="23" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="D37" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E37" s="35"/>
       <c r="F37" s="23" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B38" s="23" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E38" s="35"/>
       <c r="F38" s="23" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
     </row>
     <row r="39" spans="1:6" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="B39" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="B39" s="25" t="s">
-        <v>80</v>
-      </c>
       <c r="C39" s="25" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="D39" s="25" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E39" s="34"/>
       <c r="F39" s="25" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B40" s="23" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="D40" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E40" s="35"/>
       <c r="F40" s="23" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B41" s="23" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="D41" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E41" s="35"/>
       <c r="F41" s="23" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B42" s="23" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="D42" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E42" s="35"/>
       <c r="F42" s="23" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B43" s="23" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E43" s="35"/>
       <c r="F43" s="23" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
     </row>
     <row r="44" spans="1:6" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="24" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="B44" s="25" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C44" s="25" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="D44" s="25" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E44" s="34"/>
       <c r="F44" s="25" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B45" s="23" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="D45" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E45" s="35"/>
       <c r="F45" s="23" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="46" spans="1:6" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="24" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B46" s="25" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C46" s="25" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="D46" s="25" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E46" s="34"/>
       <c r="F46" s="25" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B47" s="23" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="D47" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E47" s="35"/>
       <c r="F47" s="23" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B48" s="23" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E48" s="35"/>
       <c r="F48" s="23" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B49" s="23" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E49" s="35"/>
       <c r="F49" s="23" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B50" s="23" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="D50" s="23" t="s">
         <v>27</v>
       </c>
       <c r="E50" s="35"/>
       <c r="F50" s="23" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B51" s="23" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E51" s="35"/>
       <c r="F51" s="23" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B52" s="23" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C52" s="23" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E52" s="35"/>
       <c r="F52" s="23" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B53" s="23" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C53" s="23" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E53" s="35"/>
       <c r="F53" s="23" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B54" s="23" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C54" s="23" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E54" s="35"/>
       <c r="F54" s="23" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B55" s="23" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C55" s="23" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="D55" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E55" s="35"/>
       <c r="F55" s="23" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B56" s="23" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C56" s="23" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E56" s="35"/>
       <c r="F56" s="23" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
@@ -4353,7 +4313,7 @@
         <v>62</v>
       </c>
       <c r="B57" s="23" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
@@ -4361,7 +4321,7 @@
         <v>23</v>
       </c>
       <c r="B58" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -4385,7 +4345,7 @@
   <sheetData>
     <row r="1" spans="1:7" s="10" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>2</v>
@@ -4408,13 +4368,13 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B2" t="s">
         <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -4422,42 +4382,42 @@
         <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="G3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B4" s="29" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C4" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B5" s="29" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B6" s="29" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C6" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B7" s="29" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -4468,66 +4428,66 @@
         <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="E8" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B9" s="29" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C9" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B10" s="29" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="C10" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B11" s="29" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="C11" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B12" s="29" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C12" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B13" s="29" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="C13" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B14" s="29" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="C14" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B15" s="29" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="C15" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
     </row>
     <row r="26" spans="9:9" x14ac:dyDescent="0.2">
@@ -4552,7 +4512,7 @@
   <sheetData>
     <row r="1" spans="1:7" s="10" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>2</v>
@@ -4592,7 +4552,7 @@
         <v>55</v>
       </c>
       <c r="C3" s="41" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -4612,7 +4572,7 @@
         <v>53</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="D4" t="s">
         <v>46</v>
@@ -4626,7 +4586,7 @@
         <v>56</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="D5" t="s">
         <v>6</v>
@@ -4655,7 +4615,7 @@
         <v>22</v>
       </c>
       <c r="F6" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="19" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fixing age group var, starting missing data analysis
</commit_message>
<xml_diff>
--- a/CleanData/DataDictionary.xlsx
+++ b/CleanData/DataDictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ainsl/Desktop/R01_Aim1H1/CleanData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E725E2C-D8E8-244A-9DDE-038F04F0C3D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8A2FBBE-52F6-E040-84C2-4C6C1AAF4D29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12600" yWindow="760" windowWidth="18380" windowHeight="17580" activeTab="1" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
+    <workbookView xWindow="3580" yWindow="3400" windowWidth="18380" windowHeight="17580" activeTab="1" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="6" r:id="rId1"/>
@@ -1758,7 +1758,7 @@
     </r>
   </si>
   <si>
-    <t>1 = "Pre-21", 2 = "21-24"</t>
+    <t>"Pre-21"  "21-24"</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Updating variables and data dictionary
</commit_message>
<xml_diff>
--- a/CleanData/DataDictionary.xlsx
+++ b/CleanData/DataDictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ainsl/Desktop/R01_Aim1H1/CleanData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8A2FBBE-52F6-E040-84C2-4C6C1AAF4D29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF0EE50-6177-CF45-91B4-1BCA7717AEC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3580" yWindow="3400" windowWidth="18380" windowHeight="17580" activeTab="1" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
+    <workbookView xWindow="12380" yWindow="760" windowWidth="18380" windowHeight="17580" activeTab="1" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="6" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="380">
   <si>
     <t>Variable</t>
   </si>
@@ -1759,6 +1759,36 @@
   </si>
   <si>
     <t>"Pre-21"  "21-24"</t>
+  </si>
+  <si>
+    <t>avg_pmk</t>
+  </si>
+  <si>
+    <t>R1485800, R2601100, R3924500, R5511000, R1485700, R2601000, R3924400, R5510900</t>
+  </si>
+  <si>
+    <t>Average parental monitoring scores for mom and dad combined from years 1999-2000</t>
+  </si>
+  <si>
+    <t>S1290100</t>
+  </si>
+  <si>
+    <t>license</t>
+  </si>
+  <si>
+    <t>Does respondent have a driver's license?</t>
+  </si>
+  <si>
+    <t>Does respondent have driver's license</t>
+  </si>
+  <si>
+    <t>Average PMK score, both mothers and fathers</t>
+  </si>
+  <si>
+    <t>avg_pmk_cat</t>
+  </si>
+  <si>
+    <t>0 = No, 1 = Yes</t>
   </si>
 </sst>
 </file>
@@ -3355,46 +3385,89 @@
       <c r="H32" s="34"/>
       <c r="I32" s="34"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A33" s="34"/>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="34"/>
-      <c r="H33" s="34"/>
-      <c r="I33" s="34"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A34" s="34"/>
-      <c r="B34" s="34"/>
-      <c r="C34" s="34"/>
-      <c r="D34" s="34"/>
-      <c r="E34" s="34"/>
-      <c r="F34" s="34"/>
-      <c r="G34" s="34"/>
+    <row r="33" spans="1:9" s="6" customFormat="1" ht="80" x14ac:dyDescent="0.2">
+      <c r="A33" s="53" t="s">
+        <v>284</v>
+      </c>
+      <c r="B33" s="54" t="s">
+        <v>93</v>
+      </c>
+      <c r="C33" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="D33" s="54" t="s">
+        <v>25</v>
+      </c>
+      <c r="E33" s="60" t="s">
+        <v>253</v>
+      </c>
+      <c r="F33" s="54" t="s">
+        <v>158</v>
+      </c>
+      <c r="G33" s="53"/>
+      <c r="H33" s="53"/>
+    </row>
+    <row r="34" spans="1:9" ht="160" x14ac:dyDescent="0.2">
+      <c r="A34" s="34" t="s">
+        <v>370</v>
+      </c>
+      <c r="B34" s="34" t="s">
+        <v>377</v>
+      </c>
+      <c r="C34" s="34" t="s">
+        <v>42</v>
+      </c>
+      <c r="D34" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="E34" s="33" t="s">
+        <v>371</v>
+      </c>
+      <c r="F34" s="34" t="s">
+        <v>306</v>
+      </c>
+      <c r="G34" s="34" t="s">
+        <v>372</v>
+      </c>
       <c r="H34" s="34"/>
       <c r="I34" s="34"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A35" s="34"/>
+    <row r="35" spans="1:9" ht="40" x14ac:dyDescent="0.2">
+      <c r="A35" s="34" t="s">
+        <v>378</v>
+      </c>
       <c r="B35" s="34"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="34"/>
+      <c r="C35" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D35" s="28" t="s">
+        <v>311</v>
+      </c>
       <c r="E35" s="34"/>
-      <c r="F35" s="34"/>
+      <c r="F35" s="34" t="s">
+        <v>306</v>
+      </c>
       <c r="G35" s="34"/>
       <c r="H35" s="34"/>
       <c r="I35" s="34"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A36" s="34"/>
-      <c r="B36" s="34"/>
+    <row r="36" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A36" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="B36" t="s">
+        <v>376</v>
+      </c>
       <c r="C36" s="34"/>
-      <c r="D36" s="34"/>
-      <c r="E36" s="34"/>
-      <c r="F36" s="34"/>
+      <c r="D36" s="34" t="s">
+        <v>379</v>
+      </c>
+      <c r="E36" t="s">
+        <v>373</v>
+      </c>
+      <c r="F36" s="34" t="s">
+        <v>306</v>
+      </c>
       <c r="G36" s="34"/>
       <c r="H36" s="34"/>
       <c r="I36" s="34"/>
@@ -5254,7 +5327,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B7A2A69-B0C6-1A43-B3A0-CA6A06B448A8}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
@@ -5572,6 +5645,17 @@
       <c r="F16" s="15"/>
       <c r="G16" s="15"/>
     </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="B17" t="s">
+        <v>373</v>
+      </c>
+      <c r="C17" t="s">
+        <v>375</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
some variable fixes and mice model
</commit_message>
<xml_diff>
--- a/CleanData/DataDictionary.xlsx
+++ b/CleanData/DataDictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ainsl/Desktop/R01_Aim1H1/CleanData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF0EE50-6177-CF45-91B4-1BCA7717AEC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E752754-7C1F-B44E-9389-494C47213C3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12380" yWindow="760" windowWidth="18380" windowHeight="17580" activeTab="1" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" firstSheet="1" activeTab="1" xr2:uid="{A5A537A6-FA63-C743-A304-1E32FC7F3E44}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="6" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="386">
   <si>
     <t>Variable</t>
   </si>
@@ -1322,9 +1322,6 @@
     <t>Income in 2002 (past-year)</t>
   </si>
   <si>
-    <t>"No", "Yes"</t>
-  </si>
-  <si>
     <t xml:space="preserve">Integer values representing the Primary Sampling Unit assignment for each respondent </t>
   </si>
   <si>
@@ -1592,48 +1589,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"M" </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">= Male, </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"F"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> = Female</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Year 1997: Among residential  </t>
     </r>
     <r>
@@ -1789,6 +1744,30 @@
   </si>
   <si>
     <t>0 = No, 1 = Yes</t>
+  </si>
+  <si>
+    <t>smoker</t>
+  </si>
+  <si>
+    <t>0 = No cigaretes reported smoking in the last 30 days, 1 = at least 1 cigarette reported smoked in the last 30 days</t>
+  </si>
+  <si>
+    <t>Binary indicator for respondent reporting smoking in the past 30 days</t>
+  </si>
+  <si>
+    <t>Created from num_cigs_02</t>
+  </si>
+  <si>
+    <t>0 = Female, 1 = Male</t>
+  </si>
+  <si>
+    <t>Maternal parenting style</t>
+  </si>
+  <si>
+    <t>Paternal parenting style</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> "Uninvolved", Permissive", Authoritarian",  Authoritative"</t>
   </si>
 </sst>
 </file>
@@ -1984,7 +1963,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -2110,11 +2089,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFADADAD"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFADADAD"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFADADAD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFADADAD"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2220,9 +2214,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2301,6 +2292,33 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2650,17 +2668,17 @@
   <sheetData>
     <row r="1" spans="1:1" ht="124" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="99" x14ac:dyDescent="0.4">
       <c r="A2" s="24" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="120" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -2670,7 +2688,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A5CC42-7E80-3145-82C3-AE1AB4759DCA}">
-  <dimension ref="A1:I123"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" style="35" customWidth="1"/>
@@ -2728,13 +2746,13 @@
         <v>30</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C3" s="25" t="s">
         <v>42</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E3" s="25" t="s">
         <v>37</v>
@@ -2743,7 +2761,7 @@
         <v>306</v>
       </c>
       <c r="G3" s="25" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="39" customFormat="1" ht="61" customHeight="1" x14ac:dyDescent="0.2">
@@ -2751,13 +2769,13 @@
         <v>38</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C4" s="25" t="s">
         <v>42</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E4" s="25" t="s">
         <v>39</v>
@@ -2766,7 +2784,7 @@
         <v>306</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="40" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.2">
@@ -2799,7 +2817,7 @@
         <v>42</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E6" s="25" t="s">
         <v>45</v>
@@ -2820,7 +2838,7 @@
         <v>25</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="E7" s="25" t="s">
         <v>45</v>
@@ -2841,7 +2859,7 @@
         <v>6</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E8" s="25" t="s">
         <v>46</v>
@@ -2862,7 +2880,7 @@
         <v>6</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E9" s="28" t="s">
         <v>47</v>
@@ -2883,7 +2901,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E10" s="28" t="s">
         <v>48</v>
@@ -2893,7 +2911,7 @@
       </c>
       <c r="G10" s="28"/>
     </row>
-    <row r="11" spans="1:7" ht="40" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="20" x14ac:dyDescent="0.2">
       <c r="A11" s="28" t="s">
         <v>15</v>
       </c>
@@ -2904,7 +2922,7 @@
         <v>25</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>355</v>
+        <v>382</v>
       </c>
       <c r="E11" s="25" t="s">
         <v>51</v>
@@ -3011,7 +3029,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>313</v>
+        <v>377</v>
       </c>
       <c r="E16" s="33" t="s">
         <v>68</v>
@@ -3021,7 +3039,7 @@
       </c>
       <c r="G16" s="33"/>
     </row>
-    <row r="17" spans="1:9" ht="40" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" ht="40" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">
         <v>258</v>
       </c>
@@ -3042,7 +3060,7 @@
       </c>
       <c r="G17" s="33"/>
     </row>
-    <row r="18" spans="1:9" ht="140" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" ht="140" x14ac:dyDescent="0.2">
       <c r="A18" s="33" t="s">
         <v>58</v>
       </c>
@@ -3063,7 +3081,7 @@
       </c>
       <c r="G18" s="33"/>
     </row>
-    <row r="19" spans="1:9" ht="40" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" ht="40" x14ac:dyDescent="0.2">
       <c r="A19" s="33" t="s">
         <v>262</v>
       </c>
@@ -3084,7 +3102,7 @@
       </c>
       <c r="G19" s="33"/>
     </row>
-    <row r="20" spans="1:9" ht="60" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" ht="60" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
         <v>59</v>
       </c>
@@ -3107,7 +3125,7 @@
       <c r="H20" s="34"/>
       <c r="I20" s="34"/>
     </row>
-    <row r="21" spans="1:9" ht="40" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" ht="40" x14ac:dyDescent="0.2">
       <c r="A21" s="33" t="s">
         <v>60</v>
       </c>
@@ -3124,7 +3142,7 @@
       <c r="H21" s="34"/>
       <c r="I21" s="34"/>
     </row>
-    <row r="22" spans="1:9" ht="100" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" ht="100" x14ac:dyDescent="0.2">
       <c r="A22" s="33" t="s">
         <v>62</v>
       </c>
@@ -3146,10 +3164,13 @@
       <c r="G22" s="33" t="s">
         <v>276</v>
       </c>
-      <c r="H22" s="34"/>
-      <c r="I22" s="34"/>
-    </row>
-    <row r="23" spans="1:9" ht="60" x14ac:dyDescent="0.2">
+      <c r="H22" s="72"/>
+      <c r="I22" s="72"/>
+      <c r="J22" s="73"/>
+      <c r="K22" s="73"/>
+      <c r="L22" s="73"/>
+    </row>
+    <row r="23" spans="1:12" ht="60" x14ac:dyDescent="0.2">
       <c r="A23" s="33" t="s">
         <v>270</v>
       </c>
@@ -3169,61 +3190,68 @@
         <v>260</v>
       </c>
       <c r="G23" s="33"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="34"/>
-    </row>
-    <row r="24" spans="1:9" ht="40" x14ac:dyDescent="0.2">
+      <c r="H23" s="72"/>
+      <c r="I23" s="72"/>
+      <c r="J23" s="73"/>
+      <c r="K23" s="73"/>
+      <c r="L23" s="73"/>
+    </row>
+    <row r="24" spans="1:12" ht="120" x14ac:dyDescent="0.2">
       <c r="A24" s="33" t="s">
+        <v>378</v>
+      </c>
+      <c r="B24" s="33" t="s">
+        <v>380</v>
+      </c>
+      <c r="C24" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="33" t="s">
+        <v>379</v>
+      </c>
+      <c r="E24" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33" t="s">
+        <v>381</v>
+      </c>
+      <c r="H24" s="72"/>
+      <c r="I24" s="72"/>
+      <c r="J24" s="73"/>
+      <c r="K24" s="73"/>
+      <c r="L24" s="73"/>
+    </row>
+    <row r="25" spans="1:12" ht="40" x14ac:dyDescent="0.2">
+      <c r="A25" s="33" t="s">
         <v>273</v>
       </c>
-      <c r="B24" s="33" t="s">
+      <c r="B25" s="33" t="s">
         <v>275</v>
       </c>
-      <c r="C24" s="33"/>
-      <c r="D24" s="33" t="s">
+      <c r="C25" s="33"/>
+      <c r="D25" s="33" t="s">
         <v>274</v>
       </c>
-      <c r="E24" s="33" t="s">
+      <c r="E25" s="33" t="s">
         <v>116</v>
       </c>
-      <c r="F24" s="33" t="s">
+      <c r="F25" s="33" t="s">
         <v>260</v>
       </c>
-      <c r="G24" s="33"/>
-      <c r="H24" s="34"/>
-      <c r="I24" s="34"/>
-    </row>
-    <row r="25" spans="1:9" ht="240" x14ac:dyDescent="0.2">
-      <c r="A25" s="28" t="s">
-        <v>335</v>
-      </c>
-      <c r="B25" s="28" t="s">
-        <v>356</v>
-      </c>
-      <c r="C25" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D25" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="E25" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="F25" s="28" t="s">
-        <v>306</v>
-      </c>
-      <c r="G25" s="28" t="s">
-        <v>336</v>
-      </c>
-      <c r="H25" s="34"/>
-      <c r="I25" s="34"/>
-    </row>
-    <row r="26" spans="1:9" ht="240" x14ac:dyDescent="0.2">
+      <c r="G25" s="33"/>
+      <c r="H25" s="72"/>
+      <c r="I25" s="72"/>
+      <c r="J25" s="73"/>
+      <c r="K25" s="73"/>
+      <c r="L25" s="73"/>
+    </row>
+    <row r="26" spans="1:12" ht="240" x14ac:dyDescent="0.2">
       <c r="A26" s="28" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="B26" s="28" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="C26" s="28" t="s">
         <v>42</v>
@@ -3232,43 +3260,51 @@
         <v>14</v>
       </c>
       <c r="E26" s="28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F26" s="28" t="s">
         <v>306</v>
       </c>
       <c r="G26" s="28" t="s">
+        <v>335</v>
+      </c>
+      <c r="H26" s="72"/>
+      <c r="I26" s="72"/>
+      <c r="J26" s="73"/>
+      <c r="K26" s="73"/>
+      <c r="L26" s="73"/>
+    </row>
+    <row r="27" spans="1:12" ht="240" x14ac:dyDescent="0.2">
+      <c r="A27" s="28" t="s">
         <v>336</v>
       </c>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
-    </row>
-    <row r="27" spans="1:9" ht="60" x14ac:dyDescent="0.2">
-      <c r="A27" s="28" t="s">
-        <v>338</v>
-      </c>
       <c r="B27" s="28" t="s">
-        <v>310</v>
+        <v>355</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>311</v>
-      </c>
-      <c r="E27" s="28"/>
+        <v>14</v>
+      </c>
+      <c r="E27" s="28" t="s">
+        <v>50</v>
+      </c>
       <c r="F27" s="28" t="s">
         <v>306</v>
       </c>
       <c r="G27" s="28" t="s">
-        <v>340</v>
-      </c>
-      <c r="H27" s="34"/>
-      <c r="I27" s="34"/>
-    </row>
-    <row r="28" spans="1:9" ht="40" x14ac:dyDescent="0.2">
+        <v>335</v>
+      </c>
+      <c r="H27" s="72"/>
+      <c r="I27" s="72"/>
+      <c r="J27" s="73"/>
+      <c r="K27" s="73"/>
+      <c r="L27" s="73"/>
+    </row>
+    <row r="28" spans="1:12" ht="60" x14ac:dyDescent="0.2">
       <c r="A28" s="28" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B28" s="28" t="s">
         <v>310</v>
@@ -3284,609 +3320,1186 @@
         <v>306</v>
       </c>
       <c r="G28" s="28" t="s">
+        <v>339</v>
+      </c>
+      <c r="H28" s="72"/>
+      <c r="I28" s="72"/>
+      <c r="J28" s="73"/>
+      <c r="K28" s="73"/>
+      <c r="L28" s="73"/>
+    </row>
+    <row r="29" spans="1:12" ht="40" x14ac:dyDescent="0.2">
+      <c r="A29" s="28" t="s">
+        <v>338</v>
+      </c>
+      <c r="B29" s="28" t="s">
         <v>310</v>
       </c>
-      <c r="H28" s="34"/>
-      <c r="I28" s="34"/>
-    </row>
-    <row r="29" spans="1:9" ht="140" x14ac:dyDescent="0.2">
-      <c r="A29" s="33" t="s">
+      <c r="C29" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" s="28" t="s">
+        <v>311</v>
+      </c>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28" t="s">
+        <v>306</v>
+      </c>
+      <c r="G29" s="28" t="s">
+        <v>310</v>
+      </c>
+      <c r="H29" s="72"/>
+      <c r="I29" s="72"/>
+      <c r="J29" s="73"/>
+      <c r="K29" s="73"/>
+      <c r="L29" s="73"/>
+    </row>
+    <row r="30" spans="1:12" ht="140" x14ac:dyDescent="0.2">
+      <c r="A30" s="33" t="s">
+        <v>340</v>
+      </c>
+      <c r="B30" s="33" t="s">
+        <v>342</v>
+      </c>
+      <c r="C30" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="D30" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" s="33" t="s">
+        <v>344</v>
+      </c>
+      <c r="F30" s="33" t="s">
+        <v>306</v>
+      </c>
+      <c r="G30" s="33" t="s">
+        <v>346</v>
+      </c>
+      <c r="H30" s="72"/>
+      <c r="I30" s="72"/>
+      <c r="J30" s="73"/>
+      <c r="K30" s="73"/>
+      <c r="L30" s="73"/>
+    </row>
+    <row r="31" spans="1:12" ht="60" x14ac:dyDescent="0.2">
+      <c r="A31" s="28" t="s">
+        <v>348</v>
+      </c>
+      <c r="B31" s="28" t="s">
+        <v>310</v>
+      </c>
+      <c r="C31" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" s="28" t="s">
+        <v>311</v>
+      </c>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28" t="s">
+        <v>306</v>
+      </c>
+      <c r="G31" s="28" t="s">
+        <v>339</v>
+      </c>
+      <c r="H31" s="72"/>
+      <c r="I31" s="72"/>
+      <c r="J31" s="73"/>
+      <c r="K31" s="73"/>
+      <c r="L31" s="73"/>
+    </row>
+    <row r="32" spans="1:12" ht="140" x14ac:dyDescent="0.2">
+      <c r="A32" s="33" t="s">
         <v>341</v>
       </c>
-      <c r="B29" s="33" t="s">
+      <c r="B32" s="33" t="s">
         <v>343</v>
       </c>
-      <c r="C29" s="33" t="s">
+      <c r="C32" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="D29" s="28" t="s">
+      <c r="D32" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="E29" s="33" t="s">
+      <c r="E32" s="33" t="s">
         <v>345</v>
       </c>
-      <c r="F29" s="33" t="s">
+      <c r="F32" s="33" t="s">
         <v>306</v>
       </c>
-      <c r="G29" s="33" t="s">
+      <c r="G32" s="33" t="s">
+        <v>346</v>
+      </c>
+      <c r="H32" s="72"/>
+      <c r="I32" s="72"/>
+      <c r="J32" s="73"/>
+      <c r="K32" s="73"/>
+      <c r="L32" s="73"/>
+    </row>
+    <row r="33" spans="1:12" ht="40" x14ac:dyDescent="0.2">
+      <c r="A33" s="28" t="s">
         <v>347</v>
       </c>
-      <c r="H29" s="34"/>
-      <c r="I29" s="34"/>
-    </row>
-    <row r="30" spans="1:9" ht="60" x14ac:dyDescent="0.2">
-      <c r="A30" s="28" t="s">
-        <v>349</v>
-      </c>
-      <c r="B30" s="28" t="s">
+      <c r="B33" s="28" t="s">
         <v>310</v>
       </c>
-      <c r="C30" s="28" t="s">
+      <c r="C33" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="D30" s="28" t="s">
+      <c r="D33" s="28" t="s">
         <v>311</v>
       </c>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28" t="s">
+      <c r="E33" s="28"/>
+      <c r="F33" s="28" t="s">
         <v>306</v>
       </c>
-      <c r="G30" s="28" t="s">
-        <v>340</v>
-      </c>
-      <c r="H30" s="34"/>
-      <c r="I30" s="34"/>
-    </row>
-    <row r="31" spans="1:9" ht="140" x14ac:dyDescent="0.2">
-      <c r="A31" s="33" t="s">
-        <v>342</v>
-      </c>
-      <c r="B31" s="33" t="s">
-        <v>344</v>
-      </c>
-      <c r="C31" s="33" t="s">
+      <c r="G33" s="28" t="s">
+        <v>310</v>
+      </c>
+      <c r="H33" s="72"/>
+      <c r="I33" s="72"/>
+      <c r="J33" s="73"/>
+      <c r="K33" s="73"/>
+      <c r="L33" s="73"/>
+    </row>
+    <row r="34" spans="1:12" s="6" customFormat="1" ht="80" x14ac:dyDescent="0.2">
+      <c r="A34" s="74" t="s">
+        <v>284</v>
+      </c>
+      <c r="B34" s="75" t="s">
+        <v>93</v>
+      </c>
+      <c r="C34" s="75" t="s">
+        <v>157</v>
+      </c>
+      <c r="D34" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34" s="76" t="s">
+        <v>253</v>
+      </c>
+      <c r="F34" s="75" t="s">
+        <v>158</v>
+      </c>
+      <c r="G34" s="74"/>
+      <c r="H34" s="74"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="15"/>
+      <c r="K34" s="15"/>
+      <c r="L34" s="15"/>
+    </row>
+    <row r="35" spans="1:12" ht="160" x14ac:dyDescent="0.2">
+      <c r="A35" s="72" t="s">
+        <v>368</v>
+      </c>
+      <c r="B35" s="72" t="s">
+        <v>375</v>
+      </c>
+      <c r="C35" s="72" t="s">
         <v>42</v>
       </c>
-      <c r="D31" s="28" t="s">
+      <c r="D35" s="72" t="s">
         <v>14</v>
       </c>
-      <c r="E31" s="33" t="s">
-        <v>346</v>
-      </c>
-      <c r="F31" s="33" t="s">
+      <c r="E35" s="33" t="s">
+        <v>369</v>
+      </c>
+      <c r="F35" s="72" t="s">
         <v>306</v>
       </c>
-      <c r="G31" s="33" t="s">
-        <v>347</v>
-      </c>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
-    </row>
-    <row r="32" spans="1:9" ht="40" x14ac:dyDescent="0.2">
-      <c r="A32" s="28" t="s">
-        <v>348</v>
-      </c>
-      <c r="B32" s="28" t="s">
-        <v>310</v>
-      </c>
-      <c r="C32" s="28" t="s">
+      <c r="G35" s="72" t="s">
+        <v>370</v>
+      </c>
+      <c r="H35" s="72"/>
+      <c r="I35" s="72"/>
+      <c r="J35" s="73"/>
+      <c r="K35" s="73"/>
+      <c r="L35" s="73"/>
+    </row>
+    <row r="36" spans="1:12" ht="40" x14ac:dyDescent="0.2">
+      <c r="A36" s="72" t="s">
+        <v>376</v>
+      </c>
+      <c r="B36" s="72"/>
+      <c r="C36" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="D32" s="28" t="s">
+      <c r="D36" s="28" t="s">
         <v>311</v>
       </c>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28" t="s">
+      <c r="E36" s="72"/>
+      <c r="F36" s="72" t="s">
         <v>306</v>
       </c>
-      <c r="G32" s="28" t="s">
-        <v>310</v>
-      </c>
-      <c r="H32" s="34"/>
-      <c r="I32" s="34"/>
-    </row>
-    <row r="33" spans="1:9" s="6" customFormat="1" ht="80" x14ac:dyDescent="0.2">
-      <c r="A33" s="53" t="s">
-        <v>284</v>
-      </c>
-      <c r="B33" s="54" t="s">
-        <v>93</v>
-      </c>
-      <c r="C33" s="54" t="s">
-        <v>157</v>
-      </c>
-      <c r="D33" s="54" t="s">
+      <c r="G36" s="72"/>
+      <c r="H36" s="72"/>
+      <c r="I36" s="72"/>
+      <c r="J36" s="73"/>
+      <c r="K36" s="73"/>
+      <c r="L36" s="73"/>
+    </row>
+    <row r="37" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A37" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>374</v>
+      </c>
+      <c r="C37" s="72"/>
+      <c r="D37" s="72" t="s">
+        <v>377</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>371</v>
+      </c>
+      <c r="F37" s="72" t="s">
+        <v>306</v>
+      </c>
+      <c r="G37" s="72"/>
+      <c r="H37" s="72"/>
+      <c r="I37" s="72"/>
+      <c r="J37" s="73"/>
+      <c r="K37" s="73"/>
+      <c r="L37" s="73"/>
+    </row>
+    <row r="38" spans="1:12" ht="48" x14ac:dyDescent="0.2">
+      <c r="A38" s="72" t="s">
+        <v>283</v>
+      </c>
+      <c r="B38" s="72" t="s">
+        <v>383</v>
+      </c>
+      <c r="C38" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="E33" s="60" t="s">
-        <v>253</v>
-      </c>
-      <c r="F33" s="54" t="s">
-        <v>158</v>
-      </c>
-      <c r="G33" s="53"/>
-      <c r="H33" s="53"/>
-    </row>
-    <row r="34" spans="1:9" ht="160" x14ac:dyDescent="0.2">
-      <c r="A34" s="34" t="s">
-        <v>370</v>
-      </c>
-      <c r="B34" s="34" t="s">
-        <v>377</v>
-      </c>
-      <c r="C34" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="D34" s="34" t="s">
-        <v>14</v>
-      </c>
-      <c r="E34" s="33" t="s">
-        <v>371</v>
-      </c>
-      <c r="F34" s="34" t="s">
-        <v>306</v>
-      </c>
-      <c r="G34" s="34" t="s">
-        <v>372</v>
-      </c>
-      <c r="H34" s="34"/>
-      <c r="I34" s="34"/>
-    </row>
-    <row r="35" spans="1:9" ht="40" x14ac:dyDescent="0.2">
-      <c r="A35" s="34" t="s">
-        <v>378</v>
-      </c>
-      <c r="B35" s="34"/>
-      <c r="C35" s="34" t="s">
+      <c r="D38" s="77" t="s">
+        <v>385</v>
+      </c>
+      <c r="E38" s="75" t="s">
+        <v>100</v>
+      </c>
+      <c r="F38" s="72" t="s">
+        <v>260</v>
+      </c>
+      <c r="G38" s="72"/>
+      <c r="H38" s="72"/>
+      <c r="I38" s="72"/>
+      <c r="J38" s="73"/>
+      <c r="K38" s="73"/>
+      <c r="L38" s="73"/>
+    </row>
+    <row r="39" spans="1:12" ht="48" x14ac:dyDescent="0.2">
+      <c r="A39" s="72" t="s">
+        <v>282</v>
+      </c>
+      <c r="B39" s="72" t="s">
+        <v>384</v>
+      </c>
+      <c r="C39" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="28" t="s">
-        <v>311</v>
-      </c>
-      <c r="E35" s="34"/>
-      <c r="F35" s="34" t="s">
-        <v>306</v>
-      </c>
-      <c r="G35" s="34"/>
-      <c r="H35" s="34"/>
-      <c r="I35" s="34"/>
-    </row>
-    <row r="36" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A36" s="12" t="s">
-        <v>374</v>
-      </c>
-      <c r="B36" t="s">
-        <v>376</v>
-      </c>
-      <c r="C36" s="34"/>
-      <c r="D36" s="34" t="s">
-        <v>379</v>
-      </c>
-      <c r="E36" t="s">
-        <v>373</v>
-      </c>
-      <c r="F36" s="34" t="s">
-        <v>306</v>
-      </c>
-      <c r="G36" s="34"/>
-      <c r="H36" s="34"/>
-      <c r="I36" s="34"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A37" s="34"/>
-      <c r="B37" s="34"/>
-      <c r="C37" s="34"/>
-      <c r="D37" s="34"/>
-      <c r="E37" s="34"/>
-      <c r="F37" s="34"/>
-      <c r="G37" s="34"/>
-      <c r="H37" s="34"/>
-      <c r="I37" s="34"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A38" s="34"/>
-      <c r="B38" s="34"/>
-      <c r="C38" s="34"/>
-      <c r="D38" s="34"/>
-      <c r="E38" s="34"/>
-      <c r="F38" s="34"/>
-      <c r="G38" s="34"/>
-      <c r="H38" s="34"/>
-      <c r="I38" s="34"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A39" s="34"/>
-      <c r="B39" s="34"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="34"/>
-      <c r="E39" s="34"/>
-      <c r="F39" s="34"/>
-      <c r="G39" s="34"/>
-      <c r="H39" s="34"/>
-      <c r="I39" s="34"/>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A40" s="34"/>
-      <c r="B40" s="34"/>
-      <c r="C40" s="34"/>
-      <c r="D40" s="34"/>
-      <c r="E40" s="34"/>
-      <c r="F40" s="34"/>
-      <c r="G40" s="34"/>
-      <c r="H40" s="34"/>
-      <c r="I40" s="34"/>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A41" s="34"/>
-      <c r="B41" s="34"/>
-      <c r="C41" s="34"/>
-      <c r="D41" s="34"/>
-      <c r="E41" s="34"/>
-      <c r="F41" s="34"/>
-      <c r="G41" s="34"/>
-      <c r="H41" s="34"/>
-      <c r="I41" s="34"/>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A42" s="34"/>
-      <c r="B42" s="34"/>
-      <c r="C42" s="34"/>
-      <c r="D42" s="34"/>
-      <c r="E42" s="34"/>
-      <c r="F42" s="34"/>
-      <c r="G42" s="34"/>
-      <c r="H42" s="34"/>
-      <c r="I42" s="34"/>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A43" s="34"/>
-      <c r="B43" s="34"/>
-      <c r="C43" s="34"/>
-      <c r="D43" s="34"/>
-      <c r="E43" s="34"/>
-      <c r="F43" s="34"/>
-      <c r="G43" s="34"/>
-      <c r="H43" s="34"/>
-      <c r="I43" s="34"/>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A44" s="34"/>
-      <c r="B44" s="34"/>
-      <c r="C44" s="34"/>
-      <c r="D44" s="34"/>
-      <c r="E44" s="34"/>
-      <c r="F44" s="34"/>
-      <c r="G44" s="34"/>
-      <c r="H44" s="34"/>
-      <c r="I44" s="34"/>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A45" s="42"/>
-      <c r="E45" s="43"/>
-      <c r="G45" s="34"/>
-      <c r="H45" s="34"/>
-      <c r="I45" s="34"/>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A46" s="42"/>
-      <c r="G46" s="34"/>
-      <c r="H46" s="34"/>
-      <c r="I46" s="34"/>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A47" s="42"/>
-      <c r="G47" s="34"/>
-      <c r="H47" s="34"/>
-      <c r="I47" s="34"/>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A48" s="42"/>
-      <c r="G48" s="34"/>
-      <c r="H48" s="34"/>
-      <c r="I48" s="34"/>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A49" s="42"/>
-      <c r="G49" s="34"/>
-      <c r="H49" s="34"/>
-      <c r="I49" s="34"/>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A50" s="42"/>
-      <c r="H50" s="34"/>
-      <c r="I50" s="34"/>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A51" s="42"/>
-      <c r="H51" s="34"/>
-      <c r="I51" s="34"/>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A52" s="42"/>
-      <c r="H52" s="34"/>
-      <c r="I52" s="34"/>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A53" s="42"/>
-      <c r="H53" s="34"/>
-      <c r="I53" s="34"/>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A54" s="42"/>
-      <c r="H54" s="44"/>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A55" s="42"/>
-      <c r="H55" s="44"/>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A56" s="42"/>
-      <c r="H56" s="44"/>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A57" s="42"/>
-      <c r="H57" s="44"/>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A58" s="42"/>
-      <c r="H58" s="44"/>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A59" s="42"/>
-      <c r="H59" s="44"/>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A60" s="42"/>
-      <c r="H60" s="44"/>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A61" s="42"/>
-      <c r="H61" s="44"/>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A62" s="42"/>
-      <c r="H62" s="44"/>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A63" s="42"/>
-      <c r="H63" s="44"/>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A64" s="42"/>
-      <c r="H64" s="44"/>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A65" s="42"/>
-      <c r="H65" s="44"/>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A66" s="42"/>
-      <c r="H66" s="44"/>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A67" s="42"/>
-      <c r="H67" s="44"/>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A68" s="42"/>
-      <c r="H68" s="44"/>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A69" s="42"/>
-      <c r="H69" s="44"/>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A70" s="42"/>
-      <c r="H70" s="44"/>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A71" s="42"/>
-      <c r="H71" s="44"/>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A72" s="42"/>
-      <c r="H72" s="44"/>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A73" s="42"/>
-      <c r="H73" s="44"/>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A74" s="42"/>
-      <c r="H74" s="44"/>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A75" s="42"/>
-      <c r="H75" s="44"/>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A76" s="42"/>
-      <c r="H76" s="44"/>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A77" s="42"/>
-      <c r="H77" s="44"/>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A78" s="42"/>
-      <c r="H78" s="44"/>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A79" s="42"/>
-      <c r="H79" s="44"/>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A80" s="42"/>
-      <c r="H80" s="44"/>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A81" s="42"/>
-      <c r="H81" s="44"/>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A82" s="42"/>
-      <c r="H82" s="44"/>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A83" s="42"/>
-      <c r="H83" s="44"/>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A84" s="42"/>
-      <c r="H84" s="44"/>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A85" s="42"/>
-      <c r="H85" s="44"/>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A86" s="42"/>
-      <c r="H86" s="44"/>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A87" s="42"/>
-      <c r="H87" s="44"/>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A88" s="42"/>
-      <c r="H88" s="44"/>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A89" s="42"/>
-      <c r="H89" s="44"/>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A90" s="42"/>
-      <c r="H90" s="44"/>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A91" s="42"/>
-      <c r="H91" s="44"/>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A92" s="42"/>
-      <c r="H92" s="44"/>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A93" s="42"/>
-      <c r="H93" s="44"/>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A94" s="42"/>
-      <c r="H94" s="44"/>
-    </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="D39" s="77" t="s">
+        <v>385</v>
+      </c>
+      <c r="E39" s="75" t="s">
+        <v>101</v>
+      </c>
+      <c r="F39" s="72" t="s">
+        <v>260</v>
+      </c>
+      <c r="G39" s="72"/>
+      <c r="H39" s="72"/>
+      <c r="I39" s="72"/>
+      <c r="J39" s="73"/>
+      <c r="K39" s="73"/>
+      <c r="L39" s="73"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A40" s="72"/>
+      <c r="B40" s="72"/>
+      <c r="C40" s="72"/>
+      <c r="D40" s="72"/>
+      <c r="E40" s="72"/>
+      <c r="F40" s="72"/>
+      <c r="G40" s="72"/>
+      <c r="H40" s="72"/>
+      <c r="I40" s="72"/>
+      <c r="J40" s="73"/>
+      <c r="K40" s="73"/>
+      <c r="L40" s="73"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A41" s="72"/>
+      <c r="B41" s="72"/>
+      <c r="C41" s="72"/>
+      <c r="D41" s="72"/>
+      <c r="E41" s="72"/>
+      <c r="F41" s="72"/>
+      <c r="G41" s="72"/>
+      <c r="H41" s="72"/>
+      <c r="I41" s="72"/>
+      <c r="J41" s="73"/>
+      <c r="K41" s="73"/>
+      <c r="L41" s="73"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A42" s="72"/>
+      <c r="B42" s="72"/>
+      <c r="C42" s="72"/>
+      <c r="D42" s="72"/>
+      <c r="E42" s="72"/>
+      <c r="F42" s="72"/>
+      <c r="G42" s="72"/>
+      <c r="H42" s="72"/>
+      <c r="I42" s="72"/>
+      <c r="J42" s="73"/>
+      <c r="K42" s="73"/>
+      <c r="L42" s="73"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A43" s="72"/>
+      <c r="B43" s="72"/>
+      <c r="C43" s="72"/>
+      <c r="D43" s="72"/>
+      <c r="E43" s="72"/>
+      <c r="F43" s="72"/>
+      <c r="G43" s="72"/>
+      <c r="H43" s="72"/>
+      <c r="I43" s="72"/>
+      <c r="J43" s="73"/>
+      <c r="K43" s="73"/>
+      <c r="L43" s="73"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A44" s="72"/>
+      <c r="B44" s="72"/>
+      <c r="C44" s="72"/>
+      <c r="D44" s="72"/>
+      <c r="E44" s="72"/>
+      <c r="F44" s="72"/>
+      <c r="G44" s="72"/>
+      <c r="H44" s="72"/>
+      <c r="I44" s="72"/>
+      <c r="J44" s="73"/>
+      <c r="K44" s="73"/>
+      <c r="L44" s="73"/>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A45" s="72"/>
+      <c r="B45" s="72"/>
+      <c r="C45" s="72"/>
+      <c r="D45" s="72"/>
+      <c r="E45" s="72"/>
+      <c r="F45" s="72"/>
+      <c r="G45" s="72"/>
+      <c r="H45" s="72"/>
+      <c r="I45" s="72"/>
+      <c r="J45" s="73"/>
+      <c r="K45" s="73"/>
+      <c r="L45" s="73"/>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A46" s="78"/>
+      <c r="B46" s="73"/>
+      <c r="C46" s="73"/>
+      <c r="D46" s="73"/>
+      <c r="E46" s="79"/>
+      <c r="F46" s="73"/>
+      <c r="G46" s="72"/>
+      <c r="H46" s="72"/>
+      <c r="I46" s="72"/>
+      <c r="J46" s="73"/>
+      <c r="K46" s="73"/>
+      <c r="L46" s="73"/>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A47" s="78"/>
+      <c r="B47" s="73"/>
+      <c r="C47" s="73"/>
+      <c r="D47" s="73"/>
+      <c r="E47" s="73"/>
+      <c r="F47" s="73"/>
+      <c r="G47" s="72"/>
+      <c r="H47" s="72"/>
+      <c r="I47" s="72"/>
+      <c r="J47" s="73"/>
+      <c r="K47" s="73"/>
+      <c r="L47" s="73"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A48" s="78"/>
+      <c r="B48" s="73"/>
+      <c r="C48" s="73"/>
+      <c r="D48" s="73"/>
+      <c r="E48" s="73"/>
+      <c r="F48" s="73"/>
+      <c r="G48" s="72"/>
+      <c r="H48" s="72"/>
+      <c r="I48" s="72"/>
+      <c r="J48" s="73"/>
+      <c r="K48" s="73"/>
+      <c r="L48" s="73"/>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A49" s="78"/>
+      <c r="B49" s="73"/>
+      <c r="C49" s="73"/>
+      <c r="D49" s="73"/>
+      <c r="E49" s="73"/>
+      <c r="F49" s="73"/>
+      <c r="G49" s="72"/>
+      <c r="H49" s="72"/>
+      <c r="I49" s="72"/>
+      <c r="J49" s="73"/>
+      <c r="K49" s="73"/>
+      <c r="L49" s="73"/>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A50" s="78"/>
+      <c r="B50" s="73"/>
+      <c r="C50" s="73"/>
+      <c r="D50" s="73"/>
+      <c r="E50" s="73"/>
+      <c r="F50" s="73"/>
+      <c r="G50" s="72"/>
+      <c r="H50" s="72"/>
+      <c r="I50" s="72"/>
+      <c r="J50" s="73"/>
+      <c r="K50" s="73"/>
+      <c r="L50" s="73"/>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A51" s="78"/>
+      <c r="B51" s="73"/>
+      <c r="C51" s="73"/>
+      <c r="D51" s="73"/>
+      <c r="E51" s="73"/>
+      <c r="F51" s="73"/>
+      <c r="G51" s="73"/>
+      <c r="H51" s="72"/>
+      <c r="I51" s="72"/>
+      <c r="J51" s="73"/>
+      <c r="K51" s="73"/>
+      <c r="L51" s="73"/>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A52" s="78"/>
+      <c r="B52" s="73"/>
+      <c r="C52" s="73"/>
+      <c r="D52" s="73"/>
+      <c r="E52" s="73"/>
+      <c r="F52" s="73"/>
+      <c r="G52" s="73"/>
+      <c r="H52" s="72"/>
+      <c r="I52" s="72"/>
+      <c r="J52" s="73"/>
+      <c r="K52" s="73"/>
+      <c r="L52" s="73"/>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A53" s="78"/>
+      <c r="B53" s="73"/>
+      <c r="C53" s="73"/>
+      <c r="D53" s="73"/>
+      <c r="E53" s="73"/>
+      <c r="F53" s="73"/>
+      <c r="G53" s="73"/>
+      <c r="H53" s="72"/>
+      <c r="I53" s="72"/>
+      <c r="J53" s="73"/>
+      <c r="K53" s="73"/>
+      <c r="L53" s="73"/>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A54" s="78"/>
+      <c r="B54" s="73"/>
+      <c r="C54" s="73"/>
+      <c r="D54" s="73"/>
+      <c r="E54" s="73"/>
+      <c r="F54" s="73"/>
+      <c r="G54" s="73"/>
+      <c r="H54" s="72"/>
+      <c r="I54" s="72"/>
+      <c r="J54" s="73"/>
+      <c r="K54" s="73"/>
+      <c r="L54" s="73"/>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A55" s="78"/>
+      <c r="B55" s="73"/>
+      <c r="C55" s="73"/>
+      <c r="D55" s="73"/>
+      <c r="E55" s="73"/>
+      <c r="F55" s="73"/>
+      <c r="G55" s="73"/>
+      <c r="H55" s="80"/>
+      <c r="I55" s="73"/>
+      <c r="J55" s="73"/>
+      <c r="K55" s="73"/>
+      <c r="L55" s="73"/>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A56" s="78"/>
+      <c r="B56" s="73"/>
+      <c r="C56" s="73"/>
+      <c r="D56" s="73"/>
+      <c r="E56" s="73"/>
+      <c r="F56" s="73"/>
+      <c r="G56" s="73"/>
+      <c r="H56" s="80"/>
+      <c r="I56" s="73"/>
+      <c r="J56" s="73"/>
+      <c r="K56" s="73"/>
+      <c r="L56" s="73"/>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A57" s="78"/>
+      <c r="B57" s="73"/>
+      <c r="C57" s="73"/>
+      <c r="D57" s="73"/>
+      <c r="E57" s="73"/>
+      <c r="F57" s="73"/>
+      <c r="G57" s="73"/>
+      <c r="H57" s="80"/>
+      <c r="I57" s="73"/>
+      <c r="J57" s="73"/>
+      <c r="K57" s="73"/>
+      <c r="L57" s="73"/>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A58" s="78"/>
+      <c r="B58" s="73"/>
+      <c r="C58" s="73"/>
+      <c r="D58" s="73"/>
+      <c r="E58" s="73"/>
+      <c r="F58" s="73"/>
+      <c r="G58" s="73"/>
+      <c r="H58" s="80"/>
+      <c r="I58" s="73"/>
+      <c r="J58" s="73"/>
+      <c r="K58" s="73"/>
+      <c r="L58" s="73"/>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A59" s="78"/>
+      <c r="B59" s="73"/>
+      <c r="C59" s="73"/>
+      <c r="D59" s="73"/>
+      <c r="E59" s="73"/>
+      <c r="F59" s="73"/>
+      <c r="G59" s="73"/>
+      <c r="H59" s="80"/>
+      <c r="I59" s="73"/>
+      <c r="J59" s="73"/>
+      <c r="K59" s="73"/>
+      <c r="L59" s="73"/>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A60" s="78"/>
+      <c r="B60" s="73"/>
+      <c r="C60" s="73"/>
+      <c r="D60" s="73"/>
+      <c r="E60" s="73"/>
+      <c r="F60" s="73"/>
+      <c r="G60" s="73"/>
+      <c r="H60" s="80"/>
+      <c r="I60" s="73"/>
+      <c r="J60" s="73"/>
+      <c r="K60" s="73"/>
+      <c r="L60" s="73"/>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A61" s="78"/>
+      <c r="B61" s="73"/>
+      <c r="C61" s="73"/>
+      <c r="D61" s="73"/>
+      <c r="E61" s="73"/>
+      <c r="F61" s="73"/>
+      <c r="G61" s="73"/>
+      <c r="H61" s="80"/>
+      <c r="I61" s="73"/>
+      <c r="J61" s="73"/>
+      <c r="K61" s="73"/>
+      <c r="L61" s="73"/>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A62" s="78"/>
+      <c r="B62" s="73"/>
+      <c r="C62" s="73"/>
+      <c r="D62" s="73"/>
+      <c r="E62" s="73"/>
+      <c r="F62" s="73"/>
+      <c r="G62" s="73"/>
+      <c r="H62" s="80"/>
+      <c r="I62" s="73"/>
+      <c r="J62" s="73"/>
+      <c r="K62" s="73"/>
+      <c r="L62" s="73"/>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A63" s="78"/>
+      <c r="B63" s="73"/>
+      <c r="C63" s="73"/>
+      <c r="D63" s="73"/>
+      <c r="E63" s="73"/>
+      <c r="F63" s="73"/>
+      <c r="G63" s="73"/>
+      <c r="H63" s="80"/>
+      <c r="I63" s="73"/>
+      <c r="J63" s="73"/>
+      <c r="K63" s="73"/>
+      <c r="L63" s="73"/>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A64" s="78"/>
+      <c r="B64" s="73"/>
+      <c r="C64" s="73"/>
+      <c r="D64" s="73"/>
+      <c r="E64" s="73"/>
+      <c r="F64" s="73"/>
+      <c r="G64" s="73"/>
+      <c r="H64" s="80"/>
+      <c r="I64" s="73"/>
+      <c r="J64" s="73"/>
+      <c r="K64" s="73"/>
+      <c r="L64" s="73"/>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A65" s="78"/>
+      <c r="B65" s="73"/>
+      <c r="C65" s="73"/>
+      <c r="D65" s="73"/>
+      <c r="E65" s="73"/>
+      <c r="F65" s="73"/>
+      <c r="G65" s="73"/>
+      <c r="H65" s="80"/>
+      <c r="I65" s="73"/>
+      <c r="J65" s="73"/>
+      <c r="K65" s="73"/>
+      <c r="L65" s="73"/>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A66" s="78"/>
+      <c r="B66" s="73"/>
+      <c r="C66" s="73"/>
+      <c r="D66" s="73"/>
+      <c r="E66" s="73"/>
+      <c r="F66" s="73"/>
+      <c r="G66" s="73"/>
+      <c r="H66" s="80"/>
+      <c r="I66" s="73"/>
+      <c r="J66" s="73"/>
+      <c r="K66" s="73"/>
+      <c r="L66" s="73"/>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A67" s="78"/>
+      <c r="B67" s="73"/>
+      <c r="C67" s="73"/>
+      <c r="D67" s="73"/>
+      <c r="E67" s="73"/>
+      <c r="F67" s="73"/>
+      <c r="G67" s="73"/>
+      <c r="H67" s="80"/>
+      <c r="I67" s="73"/>
+      <c r="J67" s="73"/>
+      <c r="K67" s="73"/>
+      <c r="L67" s="73"/>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A68" s="78"/>
+      <c r="B68" s="73"/>
+      <c r="C68" s="73"/>
+      <c r="D68" s="73"/>
+      <c r="E68" s="73"/>
+      <c r="F68" s="73"/>
+      <c r="G68" s="73"/>
+      <c r="H68" s="80"/>
+      <c r="I68" s="73"/>
+      <c r="J68" s="73"/>
+      <c r="K68" s="73"/>
+      <c r="L68" s="73"/>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A69" s="78"/>
+      <c r="B69" s="73"/>
+      <c r="C69" s="73"/>
+      <c r="D69" s="73"/>
+      <c r="E69" s="73"/>
+      <c r="F69" s="73"/>
+      <c r="G69" s="73"/>
+      <c r="H69" s="80"/>
+      <c r="I69" s="73"/>
+      <c r="J69" s="73"/>
+      <c r="K69" s="73"/>
+      <c r="L69" s="73"/>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A70" s="78"/>
+      <c r="B70" s="73"/>
+      <c r="C70" s="73"/>
+      <c r="D70" s="73"/>
+      <c r="E70" s="73"/>
+      <c r="F70" s="73"/>
+      <c r="G70" s="73"/>
+      <c r="H70" s="80"/>
+      <c r="I70" s="73"/>
+      <c r="J70" s="73"/>
+      <c r="K70" s="73"/>
+      <c r="L70" s="73"/>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A71" s="78"/>
+      <c r="B71" s="73"/>
+      <c r="C71" s="73"/>
+      <c r="D71" s="73"/>
+      <c r="E71" s="73"/>
+      <c r="F71" s="73"/>
+      <c r="G71" s="73"/>
+      <c r="H71" s="80"/>
+      <c r="I71" s="73"/>
+      <c r="J71" s="73"/>
+      <c r="K71" s="73"/>
+      <c r="L71" s="73"/>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A72" s="78"/>
+      <c r="B72" s="73"/>
+      <c r="C72" s="73"/>
+      <c r="D72" s="73"/>
+      <c r="E72" s="73"/>
+      <c r="F72" s="73"/>
+      <c r="G72" s="73"/>
+      <c r="H72" s="80"/>
+      <c r="I72" s="73"/>
+      <c r="J72" s="73"/>
+      <c r="K72" s="73"/>
+      <c r="L72" s="73"/>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A73" s="78"/>
+      <c r="B73" s="73"/>
+      <c r="C73" s="73"/>
+      <c r="D73" s="73"/>
+      <c r="E73" s="73"/>
+      <c r="F73" s="73"/>
+      <c r="G73" s="73"/>
+      <c r="H73" s="80"/>
+      <c r="I73" s="73"/>
+      <c r="J73" s="73"/>
+      <c r="K73" s="73"/>
+      <c r="L73" s="73"/>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A74" s="78"/>
+      <c r="B74" s="73"/>
+      <c r="C74" s="73"/>
+      <c r="D74" s="73"/>
+      <c r="E74" s="73"/>
+      <c r="F74" s="73"/>
+      <c r="G74" s="73"/>
+      <c r="H74" s="80"/>
+      <c r="I74" s="73"/>
+      <c r="J74" s="73"/>
+      <c r="K74" s="73"/>
+      <c r="L74" s="73"/>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A75" s="78"/>
+      <c r="B75" s="73"/>
+      <c r="C75" s="73"/>
+      <c r="D75" s="73"/>
+      <c r="E75" s="73"/>
+      <c r="F75" s="73"/>
+      <c r="G75" s="73"/>
+      <c r="H75" s="80"/>
+      <c r="I75" s="73"/>
+      <c r="J75" s="73"/>
+      <c r="K75" s="73"/>
+      <c r="L75" s="73"/>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A76" s="78"/>
+      <c r="B76" s="73"/>
+      <c r="C76" s="73"/>
+      <c r="D76" s="73"/>
+      <c r="E76" s="73"/>
+      <c r="F76" s="73"/>
+      <c r="G76" s="73"/>
+      <c r="H76" s="80"/>
+      <c r="I76" s="73"/>
+      <c r="J76" s="73"/>
+      <c r="K76" s="73"/>
+      <c r="L76" s="73"/>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A77" s="78"/>
+      <c r="B77" s="73"/>
+      <c r="C77" s="73"/>
+      <c r="D77" s="73"/>
+      <c r="E77" s="73"/>
+      <c r="F77" s="73"/>
+      <c r="G77" s="73"/>
+      <c r="H77" s="80"/>
+      <c r="I77" s="73"/>
+      <c r="J77" s="73"/>
+      <c r="K77" s="73"/>
+      <c r="L77" s="73"/>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A78" s="78"/>
+      <c r="B78" s="73"/>
+      <c r="C78" s="73"/>
+      <c r="D78" s="73"/>
+      <c r="E78" s="73"/>
+      <c r="F78" s="73"/>
+      <c r="G78" s="73"/>
+      <c r="H78" s="80"/>
+      <c r="I78" s="73"/>
+      <c r="J78" s="73"/>
+      <c r="K78" s="73"/>
+      <c r="L78" s="73"/>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A79" s="78"/>
+      <c r="B79" s="73"/>
+      <c r="C79" s="73"/>
+      <c r="D79" s="73"/>
+      <c r="E79" s="73"/>
+      <c r="F79" s="73"/>
+      <c r="G79" s="73"/>
+      <c r="H79" s="80"/>
+      <c r="I79" s="73"/>
+      <c r="J79" s="73"/>
+      <c r="K79" s="73"/>
+      <c r="L79" s="73"/>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A80" s="78"/>
+      <c r="B80" s="73"/>
+      <c r="C80" s="73"/>
+      <c r="D80" s="73"/>
+      <c r="E80" s="73"/>
+      <c r="F80" s="73"/>
+      <c r="G80" s="73"/>
+      <c r="H80" s="80"/>
+      <c r="I80" s="73"/>
+      <c r="J80" s="73"/>
+      <c r="K80" s="73"/>
+      <c r="L80" s="73"/>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A81" s="78"/>
+      <c r="B81" s="73"/>
+      <c r="C81" s="73"/>
+      <c r="D81" s="73"/>
+      <c r="E81" s="73"/>
+      <c r="F81" s="73"/>
+      <c r="G81" s="73"/>
+      <c r="H81" s="80"/>
+      <c r="I81" s="73"/>
+      <c r="J81" s="73"/>
+      <c r="K81" s="73"/>
+      <c r="L81" s="73"/>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A82" s="78"/>
+      <c r="B82" s="73"/>
+      <c r="C82" s="73"/>
+      <c r="D82" s="73"/>
+      <c r="E82" s="73"/>
+      <c r="F82" s="73"/>
+      <c r="G82" s="73"/>
+      <c r="H82" s="80"/>
+      <c r="I82" s="73"/>
+      <c r="J82" s="73"/>
+      <c r="K82" s="73"/>
+      <c r="L82" s="73"/>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A83" s="78"/>
+      <c r="B83" s="73"/>
+      <c r="C83" s="73"/>
+      <c r="D83" s="73"/>
+      <c r="E83" s="73"/>
+      <c r="F83" s="73"/>
+      <c r="G83" s="73"/>
+      <c r="H83" s="80"/>
+      <c r="I83" s="73"/>
+      <c r="J83" s="73"/>
+      <c r="K83" s="73"/>
+      <c r="L83" s="73"/>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A84" s="78"/>
+      <c r="B84" s="73"/>
+      <c r="C84" s="73"/>
+      <c r="D84" s="73"/>
+      <c r="E84" s="73"/>
+      <c r="F84" s="73"/>
+      <c r="G84" s="73"/>
+      <c r="H84" s="80"/>
+      <c r="I84" s="73"/>
+      <c r="J84" s="73"/>
+      <c r="K84" s="73"/>
+      <c r="L84" s="73"/>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A85" s="78"/>
+      <c r="B85" s="73"/>
+      <c r="C85" s="73"/>
+      <c r="D85" s="73"/>
+      <c r="E85" s="73"/>
+      <c r="F85" s="73"/>
+      <c r="G85" s="73"/>
+      <c r="H85" s="80"/>
+      <c r="I85" s="73"/>
+      <c r="J85" s="73"/>
+      <c r="K85" s="73"/>
+      <c r="L85" s="73"/>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A86" s="78"/>
+      <c r="B86" s="73"/>
+      <c r="C86" s="73"/>
+      <c r="D86" s="73"/>
+      <c r="E86" s="73"/>
+      <c r="F86" s="73"/>
+      <c r="G86" s="73"/>
+      <c r="H86" s="80"/>
+      <c r="I86" s="73"/>
+      <c r="J86" s="73"/>
+      <c r="K86" s="73"/>
+      <c r="L86" s="73"/>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A87" s="78"/>
+      <c r="B87" s="73"/>
+      <c r="C87" s="73"/>
+      <c r="D87" s="73"/>
+      <c r="E87" s="73"/>
+      <c r="F87" s="73"/>
+      <c r="G87" s="73"/>
+      <c r="H87" s="80"/>
+      <c r="I87" s="73"/>
+      <c r="J87" s="73"/>
+      <c r="K87" s="73"/>
+      <c r="L87" s="73"/>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A88" s="78"/>
+      <c r="B88" s="73"/>
+      <c r="C88" s="73"/>
+      <c r="D88" s="73"/>
+      <c r="E88" s="73"/>
+      <c r="F88" s="73"/>
+      <c r="G88" s="73"/>
+      <c r="H88" s="80"/>
+      <c r="I88" s="73"/>
+      <c r="J88" s="73"/>
+      <c r="K88" s="73"/>
+      <c r="L88" s="73"/>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A89" s="78"/>
+      <c r="B89" s="73"/>
+      <c r="C89" s="73"/>
+      <c r="D89" s="73"/>
+      <c r="E89" s="73"/>
+      <c r="F89" s="73"/>
+      <c r="G89" s="73"/>
+      <c r="H89" s="80"/>
+      <c r="I89" s="73"/>
+      <c r="J89" s="73"/>
+      <c r="K89" s="73"/>
+      <c r="L89" s="73"/>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A90" s="78"/>
+      <c r="B90" s="73"/>
+      <c r="C90" s="73"/>
+      <c r="D90" s="73"/>
+      <c r="E90" s="73"/>
+      <c r="F90" s="73"/>
+      <c r="G90" s="73"/>
+      <c r="H90" s="80"/>
+      <c r="I90" s="73"/>
+      <c r="J90" s="73"/>
+      <c r="K90" s="73"/>
+      <c r="L90" s="73"/>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A91" s="78"/>
+      <c r="B91" s="73"/>
+      <c r="C91" s="73"/>
+      <c r="D91" s="73"/>
+      <c r="E91" s="73"/>
+      <c r="F91" s="73"/>
+      <c r="G91" s="73"/>
+      <c r="H91" s="80"/>
+      <c r="I91" s="73"/>
+      <c r="J91" s="73"/>
+      <c r="K91" s="73"/>
+      <c r="L91" s="73"/>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A92" s="78"/>
+      <c r="B92" s="73"/>
+      <c r="C92" s="73"/>
+      <c r="D92" s="73"/>
+      <c r="E92" s="73"/>
+      <c r="F92" s="73"/>
+      <c r="G92" s="73"/>
+      <c r="H92" s="80"/>
+      <c r="I92" s="73"/>
+      <c r="J92" s="73"/>
+      <c r="K92" s="73"/>
+      <c r="L92" s="73"/>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A93" s="78"/>
+      <c r="B93" s="73"/>
+      <c r="C93" s="73"/>
+      <c r="D93" s="73"/>
+      <c r="E93" s="73"/>
+      <c r="F93" s="73"/>
+      <c r="G93" s="73"/>
+      <c r="H93" s="80"/>
+      <c r="I93" s="73"/>
+      <c r="J93" s="73"/>
+      <c r="K93" s="73"/>
+      <c r="L93" s="73"/>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A94" s="78"/>
+      <c r="B94" s="73"/>
+      <c r="C94" s="73"/>
+      <c r="D94" s="73"/>
+      <c r="E94" s="73"/>
+      <c r="F94" s="73"/>
+      <c r="G94" s="73"/>
+      <c r="H94" s="80"/>
+      <c r="I94" s="73"/>
+      <c r="J94" s="73"/>
+      <c r="K94" s="73"/>
+      <c r="L94" s="73"/>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A95" s="42"/>
-      <c r="H95" s="44"/>
-    </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H95" s="43"/>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" s="42"/>
-      <c r="H96" s="44"/>
+      <c r="H96" s="43"/>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A97" s="42"/>
-      <c r="H97" s="44"/>
+      <c r="H97" s="43"/>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98" s="42"/>
-      <c r="H98" s="44"/>
+      <c r="H98" s="43"/>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A99" s="42"/>
-      <c r="H99" s="44"/>
+      <c r="H99" s="43"/>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A100" s="42"/>
-      <c r="H100" s="44"/>
+      <c r="H100" s="43"/>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A101" s="42"/>
-      <c r="H101" s="44"/>
+      <c r="H101" s="43"/>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A102" s="42"/>
-      <c r="H102" s="44"/>
+      <c r="H102" s="43"/>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A103" s="42"/>
-      <c r="H103" s="44"/>
+      <c r="H103" s="43"/>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A104" s="42"/>
-      <c r="H104" s="44"/>
+      <c r="H104" s="43"/>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A105" s="42"/>
-      <c r="H105" s="44"/>
+      <c r="H105" s="43"/>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A106" s="42"/>
-      <c r="H106" s="44"/>
+      <c r="H106" s="43"/>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A107" s="42"/>
-      <c r="H107" s="44"/>
+      <c r="H107" s="43"/>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A108" s="42"/>
-      <c r="H108" s="44"/>
+      <c r="H108" s="43"/>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A109" s="42"/>
-      <c r="H109" s="44"/>
+      <c r="H109" s="43"/>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A110" s="42"/>
-      <c r="H110" s="44"/>
+      <c r="H110" s="43"/>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A111" s="42"/>
-      <c r="H111" s="44"/>
+      <c r="H111" s="43"/>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A112" s="42"/>
-      <c r="H112" s="44"/>
+      <c r="H112" s="43"/>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A113" s="42"/>
-      <c r="H113" s="44"/>
+      <c r="H113" s="43"/>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A114" s="45"/>
-      <c r="B114" s="36"/>
-      <c r="C114" s="36"/>
-      <c r="D114" s="36"/>
-      <c r="E114" s="36"/>
-      <c r="F114" s="36"/>
-      <c r="H114" s="44"/>
+      <c r="A114" s="42"/>
+      <c r="H114" s="43"/>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H115" s="44"/>
+      <c r="A115" s="44"/>
+      <c r="B115" s="36"/>
+      <c r="C115" s="36"/>
+      <c r="D115" s="36"/>
+      <c r="E115" s="36"/>
+      <c r="F115" s="36"/>
+      <c r="H115" s="43"/>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H116" s="44"/>
+      <c r="H116" s="43"/>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H117" s="44"/>
+      <c r="H117" s="43"/>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H118" s="44"/>
+      <c r="H118" s="43"/>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="G119" s="36"/>
-      <c r="H119" s="44"/>
+      <c r="H119" s="43"/>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H120" s="44"/>
+      <c r="G120" s="36"/>
+      <c r="H120" s="43"/>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H121" s="44"/>
+      <c r="H121" s="43"/>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H122" s="44"/>
+      <c r="H122" s="43"/>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H123" s="46"/>
+      <c r="H123" s="43"/>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H124" s="45"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4053,1100 +4666,1100 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" ht="23" x14ac:dyDescent="0.3">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="46" t="s">
         <v>277</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="48" t="s">
+      <c r="C1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="48" t="s">
+      <c r="D1" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="49" t="s">
+      <c r="E1" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="48" t="s">
+      <c r="F1" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="47" t="s">
+      <c r="G1" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="47"/>
+      <c r="H1" s="46"/>
     </row>
     <row r="2" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="51" t="s">
+      <c r="B2" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
     </row>
     <row r="3" spans="1:8" s="6" customFormat="1" ht="48" x14ac:dyDescent="0.2">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="53" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="54" t="s">
+      <c r="C3" s="53" t="s">
         <v>129</v>
       </c>
-      <c r="D3" s="54" t="s">
+      <c r="D3" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="55" t="s">
+      <c r="E3" s="54" t="s">
         <v>250</v>
       </c>
-      <c r="F3" s="54" t="s">
+      <c r="F3" s="53" t="s">
         <v>130</v>
       </c>
-      <c r="G3" s="53"/>
-      <c r="H3" s="53"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
     </row>
     <row r="4" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="52" t="s">
         <v>287</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="53" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="54" t="s">
+      <c r="C4" s="53" t="s">
         <v>131</v>
       </c>
-      <c r="D4" s="54" t="s">
+      <c r="D4" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="56"/>
-      <c r="F4" s="54" t="s">
+      <c r="E4" s="55"/>
+      <c r="F4" s="53" t="s">
         <v>132</v>
       </c>
-      <c r="G4" s="53"/>
-      <c r="H4" s="53" t="s">
+      <c r="G4" s="52"/>
+      <c r="H4" s="52" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="53" t="s">
+      <c r="A5" s="52" t="s">
         <v>287</v>
       </c>
-      <c r="B5" s="54" t="s">
+      <c r="B5" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="54" t="s">
+      <c r="C5" s="53" t="s">
         <v>133</v>
       </c>
-      <c r="D5" s="54" t="s">
+      <c r="D5" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="56"/>
-      <c r="F5" s="54" t="s">
+      <c r="E5" s="55"/>
+      <c r="F5" s="53" t="s">
         <v>132</v>
       </c>
-      <c r="G5" s="53"/>
-      <c r="H5" s="53"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
     </row>
     <row r="6" spans="1:8" s="6" customFormat="1" ht="32" x14ac:dyDescent="0.2">
-      <c r="A6" s="53" t="s">
+      <c r="A6" s="52" t="s">
         <v>286</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="53" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="54" t="s">
+      <c r="C6" s="53" t="s">
         <v>134</v>
       </c>
-      <c r="D6" s="54" t="s">
+      <c r="D6" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="55" t="s">
+      <c r="E6" s="54" t="s">
         <v>251</v>
       </c>
-      <c r="F6" s="54" t="s">
+      <c r="F6" s="53" t="s">
         <v>135</v>
       </c>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
     </row>
     <row r="7" spans="1:8" s="6" customFormat="1" ht="112" x14ac:dyDescent="0.2">
-      <c r="A7" s="53" t="s">
+      <c r="A7" s="52" t="s">
         <v>285</v>
       </c>
-      <c r="B7" s="54" t="s">
+      <c r="B7" s="53" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="54" t="s">
+      <c r="C7" s="53" t="s">
         <v>136</v>
       </c>
-      <c r="D7" s="54" t="s">
+      <c r="D7" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="55" t="s">
+      <c r="E7" s="54" t="s">
         <v>252</v>
       </c>
-      <c r="F7" s="54" t="s">
+      <c r="F7" s="53" t="s">
         <v>137</v>
       </c>
-      <c r="G7" s="53"/>
-      <c r="H7" s="53"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="57"/>
-      <c r="B8" s="58" t="s">
+      <c r="A8" s="56"/>
+      <c r="B8" s="57" t="s">
         <v>85</v>
       </c>
-      <c r="C8" s="58" t="s">
+      <c r="C8" s="57" t="s">
         <v>138</v>
       </c>
-      <c r="D8" s="58" t="s">
+      <c r="D8" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="59"/>
-      <c r="F8" s="58" t="s">
+      <c r="E8" s="58"/>
+      <c r="F8" s="57" t="s">
         <v>139</v>
       </c>
-      <c r="G8" s="57"/>
-      <c r="H8" s="57"/>
+      <c r="G8" s="56"/>
+      <c r="H8" s="56"/>
     </row>
     <row r="9" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="53" t="s">
+      <c r="A9" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="54" t="s">
+      <c r="B9" s="53" t="s">
         <v>86</v>
       </c>
-      <c r="C9" s="54" t="s">
+      <c r="C9" s="53" t="s">
         <v>140</v>
       </c>
-      <c r="D9" s="54" t="s">
+      <c r="D9" s="53" t="s">
         <v>141</v>
       </c>
-      <c r="E9" s="56"/>
-      <c r="F9" s="54" t="s">
+      <c r="E9" s="55"/>
+      <c r="F9" s="53" t="s">
         <v>142</v>
       </c>
-      <c r="G9" s="53" t="s">
+      <c r="G9" s="52" t="s">
         <v>238</v>
       </c>
-      <c r="H9" s="53"/>
+      <c r="H9" s="52"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="57"/>
-      <c r="B10" s="58" t="s">
+      <c r="A10" s="56"/>
+      <c r="B10" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="C10" s="58" t="s">
+      <c r="C10" s="57" t="s">
         <v>143</v>
       </c>
-      <c r="D10" s="58" t="s">
+      <c r="D10" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E10" s="59"/>
-      <c r="F10" s="58" t="s">
+      <c r="E10" s="58"/>
+      <c r="F10" s="57" t="s">
         <v>144</v>
       </c>
-      <c r="G10" s="58" t="s">
+      <c r="G10" s="57" t="s">
         <v>237</v>
       </c>
-      <c r="H10" s="57"/>
+      <c r="H10" s="56"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="57"/>
-      <c r="B11" s="58" t="s">
+      <c r="A11" s="56"/>
+      <c r="B11" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="C11" s="58" t="s">
+      <c r="C11" s="57" t="s">
         <v>145</v>
       </c>
-      <c r="D11" s="58" t="s">
+      <c r="D11" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E11" s="59"/>
-      <c r="F11" s="58" t="s">
+      <c r="E11" s="58"/>
+      <c r="F11" s="57" t="s">
         <v>146</v>
       </c>
-      <c r="G11" s="57"/>
-      <c r="H11" s="57"/>
+      <c r="G11" s="56"/>
+      <c r="H11" s="56"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="57"/>
-      <c r="B12" s="58" t="s">
+      <c r="A12" s="56"/>
+      <c r="B12" s="57" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="58" t="s">
+      <c r="C12" s="57" t="s">
         <v>147</v>
       </c>
-      <c r="D12" s="58" t="s">
+      <c r="D12" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="59"/>
-      <c r="F12" s="58" t="s">
+      <c r="E12" s="58"/>
+      <c r="F12" s="57" t="s">
         <v>148</v>
       </c>
-      <c r="G12" s="57"/>
-      <c r="H12" s="57"/>
+      <c r="G12" s="56"/>
+      <c r="H12" s="56"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="57"/>
-      <c r="B13" s="58" t="s">
+      <c r="A13" s="56"/>
+      <c r="B13" s="57" t="s">
         <v>89</v>
       </c>
-      <c r="C13" s="58" t="s">
+      <c r="C13" s="57" t="s">
         <v>149</v>
       </c>
-      <c r="D13" s="58" t="s">
+      <c r="D13" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="59"/>
-      <c r="F13" s="58" t="s">
+      <c r="E13" s="58"/>
+      <c r="F13" s="57" t="s">
         <v>150</v>
       </c>
-      <c r="G13" s="57"/>
-      <c r="H13" s="57"/>
+      <c r="G13" s="56"/>
+      <c r="H13" s="56"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="57"/>
-      <c r="B14" s="58" t="s">
+      <c r="A14" s="56"/>
+      <c r="B14" s="57" t="s">
         <v>90</v>
       </c>
-      <c r="C14" s="58" t="s">
+      <c r="C14" s="57" t="s">
         <v>151</v>
       </c>
-      <c r="D14" s="58" t="s">
+      <c r="D14" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="59"/>
-      <c r="F14" s="58" t="s">
+      <c r="E14" s="58"/>
+      <c r="F14" s="57" t="s">
         <v>152</v>
       </c>
-      <c r="G14" s="57"/>
-      <c r="H14" s="57"/>
+      <c r="G14" s="56"/>
+      <c r="H14" s="56"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="57"/>
-      <c r="B15" s="58" t="s">
+      <c r="A15" s="56"/>
+      <c r="B15" s="57" t="s">
         <v>91</v>
       </c>
-      <c r="C15" s="58" t="s">
+      <c r="C15" s="57" t="s">
         <v>153</v>
       </c>
-      <c r="D15" s="58" t="s">
+      <c r="D15" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E15" s="59"/>
-      <c r="F15" s="58" t="s">
+      <c r="E15" s="58"/>
+      <c r="F15" s="57" t="s">
         <v>154</v>
       </c>
-      <c r="G15" s="57"/>
-      <c r="H15" s="57"/>
+      <c r="G15" s="56"/>
+      <c r="H15" s="56"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="57"/>
-      <c r="B16" s="58" t="s">
+      <c r="A16" s="56"/>
+      <c r="B16" s="57" t="s">
         <v>92</v>
       </c>
-      <c r="C16" s="58" t="s">
+      <c r="C16" s="57" t="s">
         <v>155</v>
       </c>
-      <c r="D16" s="58" t="s">
+      <c r="D16" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="59"/>
-      <c r="F16" s="58" t="s">
+      <c r="E16" s="58"/>
+      <c r="F16" s="57" t="s">
         <v>156</v>
       </c>
-      <c r="G16" s="57"/>
-      <c r="H16" s="57"/>
+      <c r="G16" s="56"/>
+      <c r="H16" s="56"/>
     </row>
     <row r="17" spans="1:8" s="6" customFormat="1" ht="80" x14ac:dyDescent="0.2">
-      <c r="A17" s="53" t="s">
+      <c r="A17" s="52" t="s">
         <v>284</v>
       </c>
-      <c r="B17" s="54" t="s">
+      <c r="B17" s="53" t="s">
         <v>93</v>
       </c>
-      <c r="C17" s="54" t="s">
+      <c r="C17" s="53" t="s">
         <v>157</v>
       </c>
-      <c r="D17" s="54" t="s">
+      <c r="D17" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="60" t="s">
+      <c r="E17" s="59" t="s">
         <v>253</v>
       </c>
-      <c r="F17" s="54" t="s">
+      <c r="F17" s="53" t="s">
         <v>158</v>
       </c>
-      <c r="G17" s="53"/>
-      <c r="H17" s="53"/>
+      <c r="G17" s="52"/>
+      <c r="H17" s="52"/>
     </row>
     <row r="18" spans="1:8" s="6" customFormat="1" ht="48" x14ac:dyDescent="0.2">
-      <c r="A18" s="61" t="s">
+      <c r="A18" s="60" t="s">
         <v>281</v>
       </c>
-      <c r="B18" s="54" t="s">
+      <c r="B18" s="53" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="54" t="s">
+      <c r="C18" s="53" t="s">
         <v>159</v>
       </c>
-      <c r="D18" s="54" t="s">
+      <c r="D18" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="E18" s="56" t="s">
+      <c r="E18" s="55" t="s">
         <v>255</v>
       </c>
-      <c r="F18" s="54" t="s">
+      <c r="F18" s="53" t="s">
         <v>160</v>
       </c>
-      <c r="G18" s="53" t="s">
+      <c r="G18" s="52" t="s">
         <v>240</v>
       </c>
-      <c r="H18" s="53"/>
+      <c r="H18" s="52"/>
     </row>
     <row r="19" spans="1:8" s="6" customFormat="1" ht="48" x14ac:dyDescent="0.2">
-      <c r="A19" s="61" t="s">
+      <c r="A19" s="60" t="s">
         <v>280</v>
       </c>
-      <c r="B19" s="54" t="s">
+      <c r="B19" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="54" t="s">
+      <c r="C19" s="53" t="s">
         <v>161</v>
       </c>
-      <c r="D19" s="54" t="s">
+      <c r="D19" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="E19" s="56" t="s">
+      <c r="E19" s="55" t="s">
         <v>255</v>
       </c>
-      <c r="F19" s="54" t="s">
+      <c r="F19" s="53" t="s">
         <v>162</v>
       </c>
-      <c r="G19" s="53"/>
-      <c r="H19" s="53"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="52"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="57"/>
-      <c r="B20" s="58" t="s">
+      <c r="A20" s="56"/>
+      <c r="B20" s="57" t="s">
         <v>94</v>
       </c>
-      <c r="C20" s="58" t="s">
+      <c r="C20" s="57" t="s">
         <v>163</v>
       </c>
-      <c r="D20" s="58" t="s">
+      <c r="D20" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="59"/>
-      <c r="F20" s="58" t="s">
+      <c r="E20" s="58"/>
+      <c r="F20" s="57" t="s">
         <v>164</v>
       </c>
-      <c r="G20" s="57"/>
-      <c r="H20" s="57"/>
+      <c r="G20" s="56"/>
+      <c r="H20" s="56"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="57"/>
-      <c r="B21" s="58" t="s">
+      <c r="A21" s="56"/>
+      <c r="B21" s="57" t="s">
         <v>95</v>
       </c>
-      <c r="C21" s="58" t="s">
+      <c r="C21" s="57" t="s">
         <v>165</v>
       </c>
-      <c r="D21" s="58" t="s">
+      <c r="D21" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="59"/>
-      <c r="F21" s="58" t="s">
+      <c r="E21" s="58"/>
+      <c r="F21" s="57" t="s">
         <v>166</v>
       </c>
-      <c r="G21" s="57"/>
-      <c r="H21" s="57"/>
+      <c r="G21" s="56"/>
+      <c r="H21" s="56"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="57"/>
-      <c r="B22" s="58" t="s">
+      <c r="A22" s="56"/>
+      <c r="B22" s="57" t="s">
         <v>96</v>
       </c>
-      <c r="C22" s="58" t="s">
+      <c r="C22" s="57" t="s">
         <v>167</v>
       </c>
-      <c r="D22" s="58" t="s">
+      <c r="D22" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E22" s="59"/>
-      <c r="F22" s="58" t="s">
+      <c r="E22" s="58"/>
+      <c r="F22" s="57" t="s">
         <v>168</v>
       </c>
-      <c r="G22" s="57"/>
-      <c r="H22" s="57"/>
+      <c r="G22" s="56"/>
+      <c r="H22" s="56"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="57"/>
-      <c r="B23" s="58" t="s">
+      <c r="A23" s="56"/>
+      <c r="B23" s="57" t="s">
         <v>97</v>
       </c>
-      <c r="C23" s="58" t="s">
+      <c r="C23" s="57" t="s">
         <v>169</v>
       </c>
-      <c r="D23" s="58" t="s">
+      <c r="D23" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E23" s="59"/>
-      <c r="F23" s="58" t="s">
+      <c r="E23" s="58"/>
+      <c r="F23" s="57" t="s">
         <v>170</v>
       </c>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="57"/>
-      <c r="B24" s="58" t="s">
+      <c r="A24" s="56"/>
+      <c r="B24" s="57" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="58" t="s">
+      <c r="C24" s="57" t="s">
         <v>171</v>
       </c>
-      <c r="D24" s="58" t="s">
+      <c r="D24" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E24" s="59"/>
-      <c r="F24" s="58" t="s">
+      <c r="E24" s="58"/>
+      <c r="F24" s="57" t="s">
         <v>172</v>
       </c>
-      <c r="G24" s="57"/>
-      <c r="H24" s="57"/>
+      <c r="G24" s="56"/>
+      <c r="H24" s="56"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="57"/>
-      <c r="B25" s="58" t="s">
+      <c r="A25" s="56"/>
+      <c r="B25" s="57" t="s">
         <v>99</v>
       </c>
-      <c r="C25" s="58" t="s">
+      <c r="C25" s="57" t="s">
         <v>173</v>
       </c>
-      <c r="D25" s="58" t="s">
+      <c r="D25" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E25" s="59"/>
-      <c r="F25" s="58" t="s">
+      <c r="E25" s="58"/>
+      <c r="F25" s="57" t="s">
         <v>174</v>
       </c>
-      <c r="G25" s="57"/>
-      <c r="H25" s="57"/>
+      <c r="G25" s="56"/>
+      <c r="H25" s="56"/>
     </row>
     <row r="26" spans="1:8" s="7" customFormat="1" ht="64" x14ac:dyDescent="0.2">
-      <c r="A26" s="61" t="s">
+      <c r="A26" s="60" t="s">
         <v>283</v>
       </c>
-      <c r="B26" s="62" t="s">
+      <c r="B26" s="61" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="62" t="s">
+      <c r="C26" s="61" t="s">
         <v>175</v>
       </c>
-      <c r="D26" s="62" t="s">
+      <c r="D26" s="61" t="s">
         <v>25</v>
       </c>
-      <c r="E26" s="63" t="s">
+      <c r="E26" s="62" t="s">
         <v>254</v>
       </c>
-      <c r="F26" s="62" t="s">
+      <c r="F26" s="61" t="s">
         <v>176</v>
       </c>
-      <c r="G26" s="61" t="s">
+      <c r="G26" s="60" t="s">
         <v>239</v>
       </c>
-      <c r="H26" s="61"/>
+      <c r="H26" s="60"/>
     </row>
     <row r="27" spans="1:8" s="7" customFormat="1" ht="64" x14ac:dyDescent="0.2">
-      <c r="A27" s="61" t="s">
+      <c r="A27" s="60" t="s">
         <v>282</v>
       </c>
-      <c r="B27" s="62" t="s">
+      <c r="B27" s="61" t="s">
         <v>101</v>
       </c>
-      <c r="C27" s="62" t="s">
+      <c r="C27" s="61" t="s">
         <v>177</v>
       </c>
-      <c r="D27" s="62" t="s">
+      <c r="D27" s="61" t="s">
         <v>25</v>
       </c>
-      <c r="E27" s="63" t="s">
+      <c r="E27" s="62" t="s">
         <v>254</v>
       </c>
-      <c r="F27" s="62" t="s">
+      <c r="F27" s="61" t="s">
         <v>178</v>
       </c>
-      <c r="G27" s="61"/>
-      <c r="H27" s="61"/>
+      <c r="G27" s="60"/>
+      <c r="H27" s="60"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" s="57"/>
-      <c r="B28" s="58" t="s">
+      <c r="A28" s="56"/>
+      <c r="B28" s="57" t="s">
         <v>102</v>
       </c>
-      <c r="C28" s="58" t="s">
+      <c r="C28" s="57" t="s">
         <v>179</v>
       </c>
-      <c r="D28" s="58" t="s">
+      <c r="D28" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E28" s="59"/>
-      <c r="F28" s="58" t="s">
+      <c r="E28" s="58"/>
+      <c r="F28" s="57" t="s">
         <v>180</v>
       </c>
-      <c r="G28" s="57"/>
-      <c r="H28" s="57"/>
+      <c r="G28" s="56"/>
+      <c r="H28" s="56"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="57"/>
-      <c r="B29" s="58" t="s">
+      <c r="A29" s="56"/>
+      <c r="B29" s="57" t="s">
         <v>103</v>
       </c>
-      <c r="C29" s="58" t="s">
+      <c r="C29" s="57" t="s">
         <v>181</v>
       </c>
-      <c r="D29" s="58" t="s">
+      <c r="D29" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E29" s="59"/>
-      <c r="F29" s="58" t="s">
+      <c r="E29" s="58"/>
+      <c r="F29" s="57" t="s">
         <v>182</v>
       </c>
-      <c r="G29" s="57"/>
-      <c r="H29" s="57"/>
+      <c r="G29" s="56"/>
+      <c r="H29" s="56"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="57"/>
-      <c r="B30" s="58" t="s">
+      <c r="A30" s="56"/>
+      <c r="B30" s="57" t="s">
         <v>104</v>
       </c>
-      <c r="C30" s="58" t="s">
+      <c r="C30" s="57" t="s">
         <v>183</v>
       </c>
-      <c r="D30" s="58" t="s">
+      <c r="D30" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E30" s="59"/>
-      <c r="F30" s="58" t="s">
+      <c r="E30" s="58"/>
+      <c r="F30" s="57" t="s">
         <v>184</v>
       </c>
-      <c r="G30" s="57"/>
-      <c r="H30" s="57"/>
+      <c r="G30" s="56"/>
+      <c r="H30" s="56"/>
     </row>
     <row r="31" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="64" t="s">
+      <c r="A31" s="63" t="s">
         <v>278</v>
       </c>
-      <c r="B31" s="62" t="s">
+      <c r="B31" s="61" t="s">
         <v>65</v>
       </c>
-      <c r="C31" s="62" t="s">
+      <c r="C31" s="61" t="s">
         <v>185</v>
       </c>
-      <c r="D31" s="62" t="s">
+      <c r="D31" s="61" t="s">
         <v>141</v>
       </c>
-      <c r="E31" s="63"/>
-      <c r="F31" s="62" t="s">
+      <c r="E31" s="62"/>
+      <c r="F31" s="61" t="s">
         <v>186</v>
       </c>
-      <c r="G31" s="61"/>
-      <c r="H31" s="61"/>
+      <c r="G31" s="60"/>
+      <c r="H31" s="60"/>
     </row>
     <row r="32" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="61" t="s">
+      <c r="A32" s="60" t="s">
         <v>279</v>
       </c>
-      <c r="B32" s="62" t="s">
+      <c r="B32" s="61" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="62" t="s">
+      <c r="C32" s="61" t="s">
         <v>187</v>
       </c>
-      <c r="D32" s="62" t="s">
+      <c r="D32" s="61" t="s">
         <v>141</v>
       </c>
-      <c r="E32" s="63"/>
-      <c r="F32" s="62" t="s">
+      <c r="E32" s="62"/>
+      <c r="F32" s="61" t="s">
         <v>188</v>
       </c>
-      <c r="G32" s="61"/>
-      <c r="H32" s="61"/>
+      <c r="G32" s="60"/>
+      <c r="H32" s="60"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="57"/>
-      <c r="B33" s="58" t="s">
+      <c r="A33" s="56"/>
+      <c r="B33" s="57" t="s">
         <v>105</v>
       </c>
-      <c r="C33" s="58" t="s">
+      <c r="C33" s="57" t="s">
         <v>189</v>
       </c>
-      <c r="D33" s="58" t="s">
+      <c r="D33" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E33" s="59"/>
-      <c r="F33" s="58" t="s">
+      <c r="E33" s="58"/>
+      <c r="F33" s="57" t="s">
         <v>190</v>
       </c>
-      <c r="G33" s="57"/>
-      <c r="H33" s="57"/>
+      <c r="G33" s="56"/>
+      <c r="H33" s="56"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="57"/>
-      <c r="B34" s="58" t="s">
+      <c r="A34" s="56"/>
+      <c r="B34" s="57" t="s">
         <v>106</v>
       </c>
-      <c r="C34" s="58" t="s">
+      <c r="C34" s="57" t="s">
         <v>191</v>
       </c>
-      <c r="D34" s="58" t="s">
+      <c r="D34" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E34" s="59"/>
-      <c r="F34" s="58" t="s">
+      <c r="E34" s="58"/>
+      <c r="F34" s="57" t="s">
         <v>192</v>
       </c>
-      <c r="G34" s="57"/>
-      <c r="H34" s="57"/>
+      <c r="G34" s="56"/>
+      <c r="H34" s="56"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="57"/>
-      <c r="B35" s="58" t="s">
+      <c r="A35" s="56"/>
+      <c r="B35" s="57" t="s">
         <v>107</v>
       </c>
-      <c r="C35" s="58" t="s">
+      <c r="C35" s="57" t="s">
         <v>193</v>
       </c>
-      <c r="D35" s="58" t="s">
+      <c r="D35" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E35" s="59"/>
-      <c r="F35" s="58" t="s">
+      <c r="E35" s="58"/>
+      <c r="F35" s="57" t="s">
         <v>194</v>
       </c>
-      <c r="G35" s="57"/>
-      <c r="H35" s="57"/>
+      <c r="G35" s="56"/>
+      <c r="H35" s="56"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="57"/>
-      <c r="B36" s="58" t="s">
+      <c r="A36" s="56"/>
+      <c r="B36" s="57" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="58" t="s">
+      <c r="C36" s="57" t="s">
         <v>195</v>
       </c>
-      <c r="D36" s="58" t="s">
+      <c r="D36" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E36" s="59"/>
-      <c r="F36" s="58" t="s">
+      <c r="E36" s="58"/>
+      <c r="F36" s="57" t="s">
         <v>196</v>
       </c>
-      <c r="G36" s="57"/>
-      <c r="H36" s="57"/>
+      <c r="G36" s="56"/>
+      <c r="H36" s="56"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="57"/>
-      <c r="B37" s="58" t="s">
+      <c r="A37" s="56"/>
+      <c r="B37" s="57" t="s">
         <v>109</v>
       </c>
-      <c r="C37" s="58" t="s">
+      <c r="C37" s="57" t="s">
         <v>197</v>
       </c>
-      <c r="D37" s="58" t="s">
+      <c r="D37" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E37" s="59"/>
-      <c r="F37" s="58" t="s">
+      <c r="E37" s="58"/>
+      <c r="F37" s="57" t="s">
         <v>198</v>
       </c>
-      <c r="G37" s="57"/>
-      <c r="H37" s="57"/>
+      <c r="G37" s="56"/>
+      <c r="H37" s="56"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38" s="57"/>
-      <c r="B38" s="58" t="s">
+      <c r="A38" s="56"/>
+      <c r="B38" s="57" t="s">
         <v>66</v>
       </c>
-      <c r="C38" s="58" t="s">
+      <c r="C38" s="57" t="s">
         <v>199</v>
       </c>
-      <c r="D38" s="58" t="s">
+      <c r="D38" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E38" s="59"/>
-      <c r="F38" s="58" t="s">
+      <c r="E38" s="58"/>
+      <c r="F38" s="57" t="s">
         <v>200</v>
       </c>
-      <c r="G38" s="57"/>
-      <c r="H38" s="57"/>
+      <c r="G38" s="56"/>
+      <c r="H38" s="56"/>
     </row>
     <row r="39" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="53" t="s">
+      <c r="A39" s="52" t="s">
         <v>62</v>
       </c>
-      <c r="B39" s="54" t="s">
+      <c r="B39" s="53" t="s">
         <v>67</v>
       </c>
-      <c r="C39" s="54" t="s">
+      <c r="C39" s="53" t="s">
         <v>201</v>
       </c>
-      <c r="D39" s="54" t="s">
+      <c r="D39" s="53" t="s">
         <v>141</v>
       </c>
-      <c r="E39" s="56"/>
-      <c r="F39" s="54" t="s">
+      <c r="E39" s="55"/>
+      <c r="F39" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="G39" s="53"/>
-      <c r="H39" s="53"/>
+      <c r="G39" s="52"/>
+      <c r="H39" s="52"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="57"/>
-      <c r="B40" s="58" t="s">
+      <c r="A40" s="56"/>
+      <c r="B40" s="57" t="s">
         <v>110</v>
       </c>
-      <c r="C40" s="58" t="s">
+      <c r="C40" s="57" t="s">
         <v>203</v>
       </c>
-      <c r="D40" s="58" t="s">
+      <c r="D40" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E40" s="59"/>
-      <c r="F40" s="58" t="s">
+      <c r="E40" s="58"/>
+      <c r="F40" s="57" t="s">
         <v>204</v>
       </c>
-      <c r="G40" s="57"/>
-      <c r="H40" s="57"/>
+      <c r="G40" s="56"/>
+      <c r="H40" s="56"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" s="57"/>
-      <c r="B41" s="58" t="s">
+      <c r="A41" s="56"/>
+      <c r="B41" s="57" t="s">
         <v>111</v>
       </c>
-      <c r="C41" s="58" t="s">
+      <c r="C41" s="57" t="s">
         <v>205</v>
       </c>
-      <c r="D41" s="58" t="s">
+      <c r="D41" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E41" s="59"/>
-      <c r="F41" s="58" t="s">
+      <c r="E41" s="58"/>
+      <c r="F41" s="57" t="s">
         <v>206</v>
       </c>
-      <c r="G41" s="57"/>
-      <c r="H41" s="57"/>
+      <c r="G41" s="56"/>
+      <c r="H41" s="56"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="57"/>
-      <c r="B42" s="58" t="s">
+      <c r="A42" s="56"/>
+      <c r="B42" s="57" t="s">
         <v>112</v>
       </c>
-      <c r="C42" s="58" t="s">
+      <c r="C42" s="57" t="s">
         <v>207</v>
       </c>
-      <c r="D42" s="58" t="s">
+      <c r="D42" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E42" s="59"/>
-      <c r="F42" s="58" t="s">
+      <c r="E42" s="58"/>
+      <c r="F42" s="57" t="s">
         <v>208</v>
       </c>
-      <c r="G42" s="57"/>
-      <c r="H42" s="57"/>
+      <c r="G42" s="56"/>
+      <c r="H42" s="56"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="57"/>
-      <c r="B43" s="58" t="s">
+      <c r="A43" s="56"/>
+      <c r="B43" s="57" t="s">
         <v>113</v>
       </c>
-      <c r="C43" s="58" t="s">
+      <c r="C43" s="57" t="s">
         <v>209</v>
       </c>
-      <c r="D43" s="58" t="s">
+      <c r="D43" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E43" s="59"/>
-      <c r="F43" s="58" t="s">
+      <c r="E43" s="58"/>
+      <c r="F43" s="57" t="s">
         <v>210</v>
       </c>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
+      <c r="G43" s="56"/>
+      <c r="H43" s="56"/>
     </row>
     <row r="44" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="53" t="s">
+      <c r="A44" s="52" t="s">
         <v>270</v>
       </c>
-      <c r="B44" s="54" t="s">
+      <c r="B44" s="53" t="s">
         <v>114</v>
       </c>
-      <c r="C44" s="54" t="s">
+      <c r="C44" s="53" t="s">
         <v>211</v>
       </c>
-      <c r="D44" s="54" t="s">
+      <c r="D44" s="53" t="s">
         <v>141</v>
       </c>
-      <c r="E44" s="56"/>
-      <c r="F44" s="54" t="s">
+      <c r="E44" s="55"/>
+      <c r="F44" s="53" t="s">
         <v>212</v>
       </c>
-      <c r="G44" s="53"/>
-      <c r="H44" s="53"/>
+      <c r="G44" s="52"/>
+      <c r="H44" s="52"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A45" s="57"/>
-      <c r="B45" s="58" t="s">
+      <c r="A45" s="56"/>
+      <c r="B45" s="57" t="s">
         <v>115</v>
       </c>
-      <c r="C45" s="58" t="s">
+      <c r="C45" s="57" t="s">
         <v>213</v>
       </c>
-      <c r="D45" s="58" t="s">
+      <c r="D45" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E45" s="59"/>
-      <c r="F45" s="58" t="s">
+      <c r="E45" s="58"/>
+      <c r="F45" s="57" t="s">
         <v>214</v>
       </c>
-      <c r="G45" s="57"/>
-      <c r="H45" s="57"/>
+      <c r="G45" s="56"/>
+      <c r="H45" s="56"/>
     </row>
     <row r="46" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="53" t="s">
+      <c r="A46" s="52" t="s">
         <v>273</v>
       </c>
-      <c r="B46" s="54" t="s">
+      <c r="B46" s="53" t="s">
         <v>116</v>
       </c>
-      <c r="C46" s="54" t="s">
+      <c r="C46" s="53" t="s">
         <v>215</v>
       </c>
-      <c r="D46" s="54" t="s">
+      <c r="D46" s="53" t="s">
         <v>141</v>
       </c>
-      <c r="E46" s="56"/>
-      <c r="F46" s="54" t="s">
+      <c r="E46" s="55"/>
+      <c r="F46" s="53" t="s">
         <v>216</v>
       </c>
-      <c r="G46" s="53"/>
-      <c r="H46" s="53"/>
+      <c r="G46" s="52"/>
+      <c r="H46" s="52"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A47" s="57"/>
-      <c r="B47" s="58" t="s">
+      <c r="A47" s="56"/>
+      <c r="B47" s="57" t="s">
         <v>117</v>
       </c>
-      <c r="C47" s="58" t="s">
+      <c r="C47" s="57" t="s">
         <v>217</v>
       </c>
-      <c r="D47" s="58" t="s">
+      <c r="D47" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E47" s="59"/>
-      <c r="F47" s="58" t="s">
+      <c r="E47" s="58"/>
+      <c r="F47" s="57" t="s">
         <v>218</v>
       </c>
-      <c r="G47" s="57"/>
-      <c r="H47" s="57"/>
+      <c r="G47" s="56"/>
+      <c r="H47" s="56"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A48" s="57"/>
-      <c r="B48" s="58" t="s">
+      <c r="A48" s="56"/>
+      <c r="B48" s="57" t="s">
         <v>118</v>
       </c>
-      <c r="C48" s="58" t="s">
+      <c r="C48" s="57" t="s">
         <v>219</v>
       </c>
-      <c r="D48" s="58" t="s">
+      <c r="D48" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E48" s="59"/>
-      <c r="F48" s="58" t="s">
+      <c r="E48" s="58"/>
+      <c r="F48" s="57" t="s">
         <v>220</v>
       </c>
-      <c r="G48" s="57"/>
-      <c r="H48" s="57"/>
+      <c r="G48" s="56"/>
+      <c r="H48" s="56"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A49" s="57"/>
-      <c r="B49" s="58" t="s">
+      <c r="A49" s="56"/>
+      <c r="B49" s="57" t="s">
         <v>119</v>
       </c>
-      <c r="C49" s="58" t="s">
+      <c r="C49" s="57" t="s">
         <v>221</v>
       </c>
-      <c r="D49" s="58" t="s">
+      <c r="D49" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E49" s="59"/>
-      <c r="F49" s="58" t="s">
+      <c r="E49" s="58"/>
+      <c r="F49" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="G49" s="57"/>
-      <c r="H49" s="57"/>
+      <c r="G49" s="56"/>
+      <c r="H49" s="56"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A50" s="57"/>
-      <c r="B50" s="58" t="s">
+      <c r="A50" s="56"/>
+      <c r="B50" s="57" t="s">
         <v>120</v>
       </c>
-      <c r="C50" s="58" t="s">
+      <c r="C50" s="57" t="s">
         <v>223</v>
       </c>
-      <c r="D50" s="58" t="s">
+      <c r="D50" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="E50" s="59"/>
-      <c r="F50" s="58" t="s">
+      <c r="E50" s="58"/>
+      <c r="F50" s="57" t="s">
         <v>224</v>
       </c>
-      <c r="G50" s="57"/>
-      <c r="H50" s="57"/>
+      <c r="G50" s="56"/>
+      <c r="H50" s="56"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" s="57"/>
-      <c r="B51" s="58" t="s">
+      <c r="A51" s="56"/>
+      <c r="B51" s="57" t="s">
         <v>121</v>
       </c>
-      <c r="C51" s="58" t="s">
+      <c r="C51" s="57" t="s">
         <v>225</v>
       </c>
-      <c r="D51" s="58" t="s">
+      <c r="D51" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E51" s="59"/>
-      <c r="F51" s="58" t="s">
+      <c r="E51" s="58"/>
+      <c r="F51" s="57" t="s">
         <v>226</v>
       </c>
-      <c r="G51" s="57"/>
-      <c r="H51" s="57"/>
+      <c r="G51" s="56"/>
+      <c r="H51" s="56"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A52" s="57"/>
-      <c r="B52" s="58" t="s">
+      <c r="A52" s="56"/>
+      <c r="B52" s="57" t="s">
         <v>122</v>
       </c>
-      <c r="C52" s="58" t="s">
+      <c r="C52" s="57" t="s">
         <v>227</v>
       </c>
-      <c r="D52" s="58" t="s">
+      <c r="D52" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E52" s="59"/>
-      <c r="F52" s="58" t="s">
+      <c r="E52" s="58"/>
+      <c r="F52" s="57" t="s">
         <v>228</v>
       </c>
-      <c r="G52" s="57"/>
-      <c r="H52" s="57"/>
+      <c r="G52" s="56"/>
+      <c r="H52" s="56"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A53" s="57"/>
-      <c r="B53" s="58" t="s">
+      <c r="A53" s="56"/>
+      <c r="B53" s="57" t="s">
         <v>123</v>
       </c>
-      <c r="C53" s="58" t="s">
+      <c r="C53" s="57" t="s">
         <v>229</v>
       </c>
-      <c r="D53" s="58" t="s">
+      <c r="D53" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E53" s="59"/>
-      <c r="F53" s="58" t="s">
+      <c r="E53" s="58"/>
+      <c r="F53" s="57" t="s">
         <v>230</v>
       </c>
-      <c r="G53" s="57"/>
-      <c r="H53" s="57"/>
+      <c r="G53" s="56"/>
+      <c r="H53" s="56"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A54" s="57"/>
-      <c r="B54" s="58" t="s">
+      <c r="A54" s="56"/>
+      <c r="B54" s="57" t="s">
         <v>124</v>
       </c>
-      <c r="C54" s="58" t="s">
+      <c r="C54" s="57" t="s">
         <v>231</v>
       </c>
-      <c r="D54" s="58" t="s">
+      <c r="D54" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E54" s="59"/>
-      <c r="F54" s="58" t="s">
+      <c r="E54" s="58"/>
+      <c r="F54" s="57" t="s">
         <v>232</v>
       </c>
-      <c r="G54" s="57"/>
-      <c r="H54" s="57"/>
+      <c r="G54" s="56"/>
+      <c r="H54" s="56"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A55" s="57"/>
-      <c r="B55" s="58" t="s">
+      <c r="A55" s="56"/>
+      <c r="B55" s="57" t="s">
         <v>125</v>
       </c>
-      <c r="C55" s="58" t="s">
+      <c r="C55" s="57" t="s">
         <v>233</v>
       </c>
-      <c r="D55" s="58" t="s">
+      <c r="D55" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E55" s="59"/>
-      <c r="F55" s="58" t="s">
+      <c r="E55" s="58"/>
+      <c r="F55" s="57" t="s">
         <v>234</v>
       </c>
-      <c r="G55" s="57"/>
-      <c r="H55" s="57"/>
+      <c r="G55" s="56"/>
+      <c r="H55" s="56"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A56" s="57"/>
-      <c r="B56" s="58" t="s">
+      <c r="A56" s="56"/>
+      <c r="B56" s="57" t="s">
         <v>126</v>
       </c>
-      <c r="C56" s="58" t="s">
+      <c r="C56" s="57" t="s">
         <v>235</v>
       </c>
-      <c r="D56" s="58" t="s">
+      <c r="D56" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="E56" s="59"/>
-      <c r="F56" s="58" t="s">
+      <c r="E56" s="58"/>
+      <c r="F56" s="57" t="s">
         <v>236</v>
       </c>
-      <c r="G56" s="57"/>
-      <c r="H56" s="57"/>
+      <c r="G56" s="56"/>
+      <c r="H56" s="56"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A57" s="57" t="s">
+      <c r="A57" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="B57" s="58" t="s">
+      <c r="B57" s="57" t="s">
         <v>68</v>
       </c>
-      <c r="C57" s="57"/>
-      <c r="D57" s="57"/>
-      <c r="E57" s="65"/>
-      <c r="F57" s="57"/>
-      <c r="G57" s="57"/>
-      <c r="H57" s="57"/>
+      <c r="C57" s="56"/>
+      <c r="D57" s="56"/>
+      <c r="E57" s="64"/>
+      <c r="F57" s="56"/>
+      <c r="G57" s="56"/>
+      <c r="H57" s="56"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A58" s="57" t="s">
+      <c r="A58" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B58" s="57" t="s">
+      <c r="B58" s="56" t="s">
         <v>242</v>
       </c>
-      <c r="C58" s="57"/>
-      <c r="D58" s="57"/>
-      <c r="E58" s="65"/>
-      <c r="F58" s="57"/>
-      <c r="G58" s="57"/>
-      <c r="H58" s="57"/>
+      <c r="C58" s="56"/>
+      <c r="D58" s="56"/>
+      <c r="E58" s="64"/>
+      <c r="F58" s="56"/>
+      <c r="G58" s="56"/>
+      <c r="H58" s="56"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5248,7 +5861,7 @@
       <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="66" t="s">
+      <c r="B8" s="65" t="s">
         <v>46</v>
       </c>
       <c r="C8" s="6" t="s">
@@ -5258,7 +5871,7 @@
         <v>302</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -5341,19 +5954,19 @@
       <c r="A1" s="21" t="s">
         <v>277</v>
       </c>
-      <c r="B1" s="67" t="s">
+      <c r="B1" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="67" t="s">
+      <c r="C1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="67" t="s">
+      <c r="D1" s="66" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="67" t="s">
+      <c r="E1" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="67" t="s">
+      <c r="F1" s="66" t="s">
         <v>1</v>
       </c>
       <c r="G1" s="21" t="s">
@@ -5376,13 +5989,13 @@
       <c r="G2" s="15"/>
     </row>
     <row r="3" spans="1:7" ht="102" x14ac:dyDescent="0.2">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="68" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="70" t="s">
+      <c r="C3" s="69" t="s">
         <v>308</v>
       </c>
       <c r="D3" s="15" t="s">
@@ -5397,13 +6010,13 @@
       <c r="G3" s="15"/>
     </row>
     <row r="4" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="67" t="s">
         <v>40</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="69" t="s">
         <v>305</v>
       </c>
       <c r="D4" s="15" t="s">
@@ -5420,7 +6033,7 @@
       <c r="B5" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="70" t="s">
+      <c r="C5" s="69" t="s">
         <v>309</v>
       </c>
       <c r="D5" s="15" t="s">
@@ -5435,7 +6048,7 @@
       <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" ht="128" x14ac:dyDescent="0.2">
-      <c r="A6" s="68" t="s">
+      <c r="A6" s="67" t="s">
         <v>18</v>
       </c>
       <c r="B6" s="12" t="s">
@@ -5463,13 +6076,13 @@
         <v>37</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D7" s="25" t="s">
         <v>42</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F7" s="15"/>
       <c r="G7" s="15"/>
@@ -5482,26 +6095,26 @@
         <v>39</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D8" s="25" t="s">
         <v>42</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
     </row>
     <row r="9" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
-        <v>321</v>
-      </c>
-      <c r="B9" s="71" t="s">
+        <v>320</v>
+      </c>
+      <c r="B9" s="70" t="s">
         <v>50</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="D9" s="28" t="s">
         <v>42</v>
@@ -5514,13 +6127,13 @@
     </row>
     <row r="10" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="B10" s="71" t="s">
-        <v>329</v>
+        <v>321</v>
+      </c>
+      <c r="B10" s="70" t="s">
+        <v>328</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="D10" s="28" t="s">
         <v>42</v>
@@ -5533,13 +6146,13 @@
     </row>
     <row r="11" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
-        <v>323</v>
-      </c>
-      <c r="B11" s="71" t="s">
-        <v>331</v>
-      </c>
-      <c r="C11" s="72" t="s">
-        <v>361</v>
+        <v>322</v>
+      </c>
+      <c r="B11" s="70" t="s">
+        <v>330</v>
+      </c>
+      <c r="C11" s="71" t="s">
+        <v>359</v>
       </c>
       <c r="D11" s="28" t="s">
         <v>42</v>
@@ -5552,13 +6165,13 @@
     </row>
     <row r="12" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
-        <v>324</v>
-      </c>
-      <c r="B12" s="71" t="s">
-        <v>333</v>
-      </c>
-      <c r="C12" s="72" t="s">
-        <v>362</v>
+        <v>323</v>
+      </c>
+      <c r="B12" s="70" t="s">
+        <v>332</v>
+      </c>
+      <c r="C12" s="71" t="s">
+        <v>360</v>
       </c>
       <c r="D12" s="28" t="s">
         <v>42</v>
@@ -5571,13 +6184,13 @@
     </row>
     <row r="13" spans="1:7" ht="20" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
-        <v>325</v>
-      </c>
-      <c r="B13" s="71" t="s">
+        <v>324</v>
+      </c>
+      <c r="B13" s="70" t="s">
         <v>49</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="D13" s="28" t="s">
         <v>42</v>
@@ -5590,13 +6203,13 @@
     </row>
     <row r="14" spans="1:7" ht="20" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
-        <v>326</v>
-      </c>
-      <c r="B14" s="71" t="s">
-        <v>330</v>
+        <v>325</v>
+      </c>
+      <c r="B14" s="70" t="s">
+        <v>329</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D14" s="28" t="s">
         <v>42</v>
@@ -5609,13 +6222,13 @@
     </row>
     <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
-        <v>327</v>
-      </c>
-      <c r="B15" s="71" t="s">
-        <v>332</v>
+        <v>326</v>
+      </c>
+      <c r="B15" s="70" t="s">
+        <v>331</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="D15" s="28" t="s">
         <v>42</v>
@@ -5628,13 +6241,13 @@
     </row>
     <row r="16" spans="1:7" ht="20" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
-        <v>328</v>
-      </c>
-      <c r="B16" s="71" t="s">
-        <v>334</v>
+        <v>327</v>
+      </c>
+      <c r="B16" s="70" t="s">
+        <v>333</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D16" s="28" t="s">
         <v>42</v>
@@ -5647,13 +6260,13 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="12" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B17" t="s">
+        <v>371</v>
+      </c>
+      <c r="C17" t="s">
         <v>373</v>
-      </c>
-      <c r="C17" t="s">
-        <v>375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>